<commit_message>
succesfully running scenarios for rothc. Checking residues monthly are running correctly
</commit_message>
<xml_diff>
--- a/data/crops/rothc_support/annual_crops_rothc_scenarios_rainfed_FAOGAEZ.xlsx
+++ b/data/crops/rothc_support/annual_crops_rothc_scenarios_rainfed_FAOGAEZ.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://worldwildlifefund-my.sharepoint.com/personal/cristobal_loyola_wwfus_org/Documents/Documents/203. Python projects/SBTN_Test/data/crops/rothc_support/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="148" documentId="8_{170725B8-9B34-4153-8604-E86F3A22CBBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3157047F-C89D-49A2-8408-3BD6DEA30C50}"/>
+  <xr:revisionPtr revIDLastSave="158" documentId="8_{170725B8-9B34-4153-8604-E86F3A22CBBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{91E1FFCD-C147-47A4-AAD0-87F58580F299}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{6F94B64D-243B-49DA-AE87-045B34BFAB0F}"/>
   </bookViews>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2492" uniqueCount="609">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2534" uniqueCount="613">
   <si>
     <t>crop_name</t>
   </si>
@@ -1888,13 +1888,72 @@
   </si>
   <si>
     <t>C:\Users\loyola\OneDrive - World Wildlife Fund, Inc\Documents\203. Python projects\SBTN_Test\data\land_use\FAO_GAEZ/lu_gaez_Sugar beet_rf.tif</t>
+  </si>
+  <si>
+    <t>outlier_strategy</t>
+  </si>
+  <si>
+    <r>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="7"/>
+        <color rgb="FFFF9E64"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>1.0</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="7"/>
+        <color rgb="FF89DDFF"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>,</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="7"/>
+        <color rgb="FFA9B1D6"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="7"/>
+        <color rgb="FFFF9E64"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>99.0</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="7"/>
+        <color rgb="FF89DDFF"/>
+        <rFont val="Consolas"/>
+        <family val="3"/>
+      </rPr>
+      <t>)</t>
+    </r>
+  </si>
+  <si>
+    <t>log_winsor</t>
+  </si>
+  <si>
+    <t>percentile_bound</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1909,6 +1968,24 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="7"/>
+      <color rgb="FFA9B1D6"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="7"/>
+      <color rgb="FF89DDFF"/>
+      <name val="Consolas"/>
+      <family val="3"/>
+    </font>
+    <font>
+      <sz val="7"/>
+      <color rgb="FFFF9E64"/>
+      <name val="Consolas"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="3">
@@ -1970,20 +2047,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2068,13 +2141,13 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{55C0E0B5-21B5-4E14-A12B-9F865E445D80}" name="annual_crops_FAO_GAEZ_data_path" displayName="annual_crops_FAO_GAEZ_data_path" ref="A1:G35" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:G35" xr:uid="{55C0E0B5-21B5-4E14-A12B-9F865E445D80}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{D2CDBE54-7DFE-495A-8C47-0C4F483A9A36}" uniqueName="1" name="crop_name" queryTableFieldId="1" dataDxfId="6"/>
-    <tableColumn id="2" xr3:uid="{36A2073A-17B5-424E-891A-56660DA50771}" uniqueName="2" name="crop_type" queryTableFieldId="2" dataDxfId="5"/>
-    <tableColumn id="3" xr3:uid="{12B2EC26-9574-4C81-AE25-5FBA0E4D7A76}" uniqueName="3" name="crop_practice_string" queryTableFieldId="3" dataDxfId="4"/>
-    <tableColumn id="4" xr3:uid="{A981D2A3-6A91-43D2-B7DC-9361B9A8F20A}" uniqueName="4" name="lu_path" queryTableFieldId="4" dataDxfId="3"/>
-    <tableColumn id="5" xr3:uid="{B4B4350A-23D3-4A7F-98E1-A6388FB4A1FD}" uniqueName="5" name="pet_path" queryTableFieldId="5" dataDxfId="2"/>
-    <tableColumn id="6" xr3:uid="{4DAE9F00-2A7F-4200-ADAF-52CB5C9B1A19}" uniqueName="6" name="irr_path" queryTableFieldId="6" dataDxfId="1"/>
-    <tableColumn id="7" xr3:uid="{EB04586B-94DF-4D65-A607-26B04ABC6F8D}" uniqueName="7" name="plantcover_path" queryTableFieldId="7" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{D2CDBE54-7DFE-495A-8C47-0C4F483A9A36}" uniqueName="1" name="crop_name" queryTableFieldId="1" dataDxfId="10"/>
+    <tableColumn id="2" xr3:uid="{36A2073A-17B5-424E-891A-56660DA50771}" uniqueName="2" name="crop_type" queryTableFieldId="2" dataDxfId="9"/>
+    <tableColumn id="3" xr3:uid="{12B2EC26-9574-4C81-AE25-5FBA0E4D7A76}" uniqueName="3" name="crop_practice_string" queryTableFieldId="3" dataDxfId="8"/>
+    <tableColumn id="4" xr3:uid="{A981D2A3-6A91-43D2-B7DC-9361B9A8F20A}" uniqueName="4" name="lu_path" queryTableFieldId="4" dataDxfId="7"/>
+    <tableColumn id="5" xr3:uid="{B4B4350A-23D3-4A7F-98E1-A6388FB4A1FD}" uniqueName="5" name="pet_path" queryTableFieldId="5" dataDxfId="6"/>
+    <tableColumn id="6" xr3:uid="{4DAE9F00-2A7F-4200-ADAF-52CB5C9B1A19}" uniqueName="6" name="irr_path" queryTableFieldId="6" dataDxfId="5"/>
+    <tableColumn id="7" xr3:uid="{EB04586B-94DF-4D65-A607-26B04ABC6F8D}" uniqueName="7" name="plantcover_path" queryTableFieldId="7" dataDxfId="4"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2084,10 +2157,10 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{D4138EED-881E-411A-BC79-FB457DA6FC5D}" name="faogaez_yield_file_index__2" displayName="faogaez_yield_file_index__2" ref="A1:D38" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:D38" xr:uid="{D4138EED-881E-411A-BC79-FB457DA6FC5D}"/>
   <tableColumns count="4">
-    <tableColumn id="5" xr3:uid="{3E605F29-4B62-42C4-B46E-4709285BBD84}" uniqueName="5" name="crop_name" queryTableFieldId="5" dataDxfId="10"/>
-    <tableColumn id="8" xr3:uid="{6E0A94BC-5E44-4F12-9A16-8BC520BDE6DA}" uniqueName="8" name="Total" queryTableFieldId="8" dataDxfId="7"/>
-    <tableColumn id="6" xr3:uid="{1F96D6F4-19CF-41F4-8F71-F7F45D3012FC}" uniqueName="6" name="Irrigated" queryTableFieldId="6" dataDxfId="9"/>
-    <tableColumn id="7" xr3:uid="{6C72B11B-83D3-4D0C-B671-13558C118237}" uniqueName="7" name="Rainfed" queryTableFieldId="7" dataDxfId="8"/>
+    <tableColumn id="5" xr3:uid="{3E605F29-4B62-42C4-B46E-4709285BBD84}" uniqueName="5" name="crop_name" queryTableFieldId="5" dataDxfId="3"/>
+    <tableColumn id="8" xr3:uid="{6E0A94BC-5E44-4F12-9A16-8BC520BDE6DA}" uniqueName="8" name="Total" queryTableFieldId="8" dataDxfId="2"/>
+    <tableColumn id="6" xr3:uid="{1F96D6F4-19CF-41F4-8F71-F7F45D3012FC}" uniqueName="6" name="Irrigated" queryTableFieldId="6" dataDxfId="1"/>
+    <tableColumn id="7" xr3:uid="{6C72B11B-83D3-4D0C-B671-13558C118237}" uniqueName="7" name="Rainfed" queryTableFieldId="7" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2410,7 +2483,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A1821CC5-2977-4A1A-B60B-8C004F05C4AF}">
-  <dimension ref="A1:V21"/>
+  <dimension ref="A1:X21"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11.36328125" bestFit="1" customWidth="1"/>
@@ -2420,9 +2493,11 @@
     <col min="6" max="6" width="18.26953125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="49.36328125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="27.1796875" customWidth="1"/>
+    <col min="23" max="23" width="13.81640625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="16.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -2489,8 +2564,14 @@
       <c r="V1" s="2" t="s">
         <v>477</v>
       </c>
-    </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="W1" s="2" t="s">
+        <v>609</v>
+      </c>
+      <c r="X1" s="8" t="s">
+        <v>612</v>
+      </c>
+    </row>
+    <row r="2" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>15</v>
       </c>
@@ -2531,16 +2612,16 @@
       <c r="P2">
         <v>100</v>
       </c>
-      <c r="Q2" s="8" t="s">
+      <c r="Q2" s="6" t="s">
         <v>344</v>
       </c>
-      <c r="R2" s="7" t="s">
+      <c r="R2" s="3" t="s">
         <v>345</v>
       </c>
-      <c r="S2" s="7" t="s">
+      <c r="S2" s="3" t="s">
         <v>343</v>
       </c>
-      <c r="T2" s="8" t="s">
+      <c r="T2" s="6" t="s">
         <v>344</v>
       </c>
       <c r="U2" t="b">
@@ -2549,8 +2630,14 @@
       <c r="V2" t="s">
         <v>478</v>
       </c>
-    </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="W2" t="s">
+        <v>611</v>
+      </c>
+      <c r="X2" t="s">
+        <v>610</v>
+      </c>
+    </row>
+    <row r="3" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>15</v>
       </c>
@@ -2591,16 +2678,16 @@
       <c r="P3">
         <v>100</v>
       </c>
-      <c r="Q3" s="8" t="s">
+      <c r="Q3" s="6" t="s">
         <v>344</v>
       </c>
-      <c r="R3" s="7" t="s">
+      <c r="R3" s="3" t="s">
         <v>345</v>
       </c>
-      <c r="S3" s="7" t="s">
+      <c r="S3" s="3" t="s">
         <v>343</v>
       </c>
-      <c r="T3" s="8" t="s">
+      <c r="T3" s="6" t="s">
         <v>344</v>
       </c>
       <c r="U3" t="b">
@@ -2609,8 +2696,14 @@
       <c r="V3" t="s">
         <v>478</v>
       </c>
-    </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="W3" t="s">
+        <v>611</v>
+      </c>
+      <c r="X3" t="s">
+        <v>610</v>
+      </c>
+    </row>
+    <row r="4" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>18</v>
       </c>
@@ -2639,10 +2732,10 @@
       <c r="I4" s="3" t="s">
         <v>480</v>
       </c>
-      <c r="J4" s="9" t="s">
+      <c r="J4" s="6" t="s">
         <v>481</v>
       </c>
-      <c r="K4" s="9"/>
+      <c r="K4" s="6"/>
       <c r="N4" t="b">
         <v>0</v>
       </c>
@@ -2652,26 +2745,32 @@
       <c r="P4">
         <v>100</v>
       </c>
-      <c r="Q4" s="11" t="s">
+      <c r="Q4" s="5" t="s">
         <v>360</v>
       </c>
-      <c r="R4" s="10" t="s">
+      <c r="R4" s="4" t="s">
         <v>361</v>
       </c>
-      <c r="S4" s="10" t="s">
+      <c r="S4" s="4" t="s">
         <v>359</v>
       </c>
-      <c r="T4" s="11" t="s">
+      <c r="T4" s="5" t="s">
         <v>360</v>
       </c>
       <c r="U4" t="b">
         <v>1</v>
       </c>
-      <c r="V4" s="12" t="s">
+      <c r="V4" s="7" t="s">
         <v>478</v>
       </c>
-    </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="W4" t="s">
+        <v>611</v>
+      </c>
+      <c r="X4" t="s">
+        <v>610</v>
+      </c>
+    </row>
+    <row r="5" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>19</v>
       </c>
@@ -2712,26 +2811,32 @@
       <c r="P5">
         <v>100</v>
       </c>
-      <c r="Q5" s="11" t="s">
+      <c r="Q5" s="5" t="s">
         <v>366</v>
       </c>
-      <c r="R5" s="10" t="s">
+      <c r="R5" s="4" t="s">
         <v>367</v>
       </c>
-      <c r="S5" s="10" t="s">
+      <c r="S5" s="4" t="s">
         <v>365</v>
       </c>
-      <c r="T5" s="11" t="s">
+      <c r="T5" s="5" t="s">
         <v>366</v>
       </c>
       <c r="U5" t="b">
         <v>1</v>
       </c>
-      <c r="V5" s="12" t="s">
+      <c r="V5" s="7" t="s">
         <v>478</v>
       </c>
-    </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="W5" t="s">
+        <v>611</v>
+      </c>
+      <c r="X5" t="s">
+        <v>610</v>
+      </c>
+    </row>
+    <row r="6" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>20</v>
       </c>
@@ -2760,7 +2865,7 @@
       <c r="I6" s="3" t="s">
         <v>486</v>
       </c>
-      <c r="J6" s="9" t="s">
+      <c r="J6" s="6" t="s">
         <v>487</v>
       </c>
       <c r="N6" t="b">
@@ -2772,26 +2877,32 @@
       <c r="P6">
         <v>100</v>
       </c>
-      <c r="Q6" s="8" t="s">
+      <c r="Q6" s="6" t="s">
         <v>369</v>
       </c>
-      <c r="R6" s="7" t="s">
+      <c r="R6" s="3" t="s">
         <v>370</v>
       </c>
-      <c r="S6" s="7" t="s">
+      <c r="S6" s="3" t="s">
         <v>368</v>
       </c>
-      <c r="T6" s="8" t="s">
+      <c r="T6" s="6" t="s">
         <v>369</v>
       </c>
       <c r="U6" t="b">
         <v>1</v>
       </c>
-      <c r="V6" s="12" t="s">
+      <c r="V6" s="7" t="s">
         <v>478</v>
       </c>
-    </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="W6" t="s">
+        <v>611</v>
+      </c>
+      <c r="X6" t="s">
+        <v>610</v>
+      </c>
+    </row>
+    <row r="7" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>20</v>
       </c>
@@ -2820,7 +2931,7 @@
       <c r="I7" s="3" t="s">
         <v>486</v>
       </c>
-      <c r="J7" s="9" t="s">
+      <c r="J7" s="6" t="s">
         <v>487</v>
       </c>
       <c r="N7" t="b">
@@ -2832,26 +2943,32 @@
       <c r="P7">
         <v>100</v>
       </c>
-      <c r="Q7" s="8" t="s">
+      <c r="Q7" s="6" t="s">
         <v>369</v>
       </c>
-      <c r="R7" s="7" t="s">
+      <c r="R7" s="3" t="s">
         <v>370</v>
       </c>
-      <c r="S7" s="7" t="s">
+      <c r="S7" s="3" t="s">
         <v>368</v>
       </c>
-      <c r="T7" s="8" t="s">
+      <c r="T7" s="6" t="s">
         <v>369</v>
       </c>
       <c r="U7" t="b">
         <v>1</v>
       </c>
-      <c r="V7" s="12" t="s">
+      <c r="V7" s="7" t="s">
         <v>478</v>
       </c>
-    </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="W7" t="s">
+        <v>611</v>
+      </c>
+      <c r="X7" t="s">
+        <v>610</v>
+      </c>
+    </row>
+    <row r="8" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>22</v>
       </c>
@@ -2892,26 +3009,32 @@
       <c r="P8">
         <v>100</v>
       </c>
-      <c r="Q8" s="11" t="s">
+      <c r="Q8" s="5" t="s">
         <v>463</v>
       </c>
-      <c r="R8" s="10" t="s">
+      <c r="R8" s="4" t="s">
         <v>464</v>
       </c>
-      <c r="S8" s="10" t="s">
+      <c r="S8" s="4" t="s">
         <v>462</v>
       </c>
-      <c r="T8" s="11" t="s">
+      <c r="T8" s="5" t="s">
         <v>463</v>
       </c>
       <c r="U8" t="b">
         <v>1</v>
       </c>
-      <c r="V8" s="12" t="s">
+      <c r="V8" s="7" t="s">
         <v>478</v>
       </c>
-    </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="W8" t="s">
+        <v>611</v>
+      </c>
+      <c r="X8" t="s">
+        <v>610</v>
+      </c>
+    </row>
+    <row r="9" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>23</v>
       </c>
@@ -2940,7 +3063,7 @@
       <c r="I9" s="3" t="s">
         <v>492</v>
       </c>
-      <c r="J9" s="9" t="s">
+      <c r="J9" s="6" t="s">
         <v>493</v>
       </c>
       <c r="N9" t="b">
@@ -2952,26 +3075,32 @@
       <c r="P9">
         <v>100</v>
       </c>
-      <c r="Q9" s="11" t="s">
+      <c r="Q9" s="5" t="s">
         <v>378</v>
       </c>
-      <c r="R9" s="10" t="s">
+      <c r="R9" s="4" t="s">
         <v>379</v>
       </c>
-      <c r="S9" s="10" t="s">
+      <c r="S9" s="4" t="s">
         <v>377</v>
       </c>
-      <c r="T9" s="11" t="s">
+      <c r="T9" s="5" t="s">
         <v>378</v>
       </c>
       <c r="U9" t="b">
         <v>1</v>
       </c>
-      <c r="V9" s="12" t="s">
+      <c r="V9" s="7" t="s">
         <v>478</v>
       </c>
-    </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="W9" t="s">
+        <v>611</v>
+      </c>
+      <c r="X9" t="s">
+        <v>610</v>
+      </c>
+    </row>
+    <row r="10" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>23</v>
       </c>
@@ -3000,7 +3129,7 @@
       <c r="I10" s="3" t="s">
         <v>492</v>
       </c>
-      <c r="J10" s="9" t="s">
+      <c r="J10" s="6" t="s">
         <v>493</v>
       </c>
       <c r="N10" t="b">
@@ -3012,26 +3141,32 @@
       <c r="P10">
         <v>100</v>
       </c>
-      <c r="Q10" s="11" t="s">
+      <c r="Q10" s="5" t="s">
         <v>378</v>
       </c>
-      <c r="R10" s="10" t="s">
+      <c r="R10" s="4" t="s">
         <v>379</v>
       </c>
-      <c r="S10" s="10" t="s">
+      <c r="S10" s="4" t="s">
         <v>377</v>
       </c>
-      <c r="T10" s="11" t="s">
+      <c r="T10" s="5" t="s">
         <v>378</v>
       </c>
       <c r="U10" t="b">
         <v>1</v>
       </c>
-      <c r="V10" s="12" t="s">
+      <c r="V10" s="7" t="s">
         <v>478</v>
       </c>
-    </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="W10" t="s">
+        <v>611</v>
+      </c>
+      <c r="X10" t="s">
+        <v>610</v>
+      </c>
+    </row>
+    <row r="11" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>24</v>
       </c>
@@ -3072,26 +3207,32 @@
       <c r="P11">
         <v>100</v>
       </c>
-      <c r="Q11" s="8" t="s">
+      <c r="Q11" s="6" t="s">
         <v>375</v>
       </c>
-      <c r="R11" s="7" t="s">
+      <c r="R11" s="3" t="s">
         <v>376</v>
       </c>
-      <c r="S11" s="7" t="s">
+      <c r="S11" s="3" t="s">
         <v>374</v>
       </c>
-      <c r="T11" s="8" t="s">
+      <c r="T11" s="6" t="s">
         <v>375</v>
       </c>
       <c r="U11" t="b">
         <v>1</v>
       </c>
-      <c r="V11" s="12" t="s">
+      <c r="V11" s="7" t="s">
         <v>478</v>
       </c>
-    </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="W11" t="s">
+        <v>611</v>
+      </c>
+      <c r="X11" t="s">
+        <v>610</v>
+      </c>
+    </row>
+    <row r="12" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>25</v>
       </c>
@@ -3114,13 +3255,13 @@
         <f t="shared" si="0"/>
         <v>RothC results for year 2030 for Sorghum_rf_ron in ton C/ha</v>
       </c>
-      <c r="H12" s="10" t="s">
+      <c r="H12" s="4" t="s">
         <v>600</v>
       </c>
-      <c r="I12" s="10" t="s">
+      <c r="I12" s="4" t="s">
         <v>601</v>
       </c>
-      <c r="J12" s="11" t="s">
+      <c r="J12" s="5" t="s">
         <v>603</v>
       </c>
       <c r="N12" t="b">
@@ -3132,26 +3273,32 @@
       <c r="P12">
         <v>100</v>
       </c>
-      <c r="Q12" s="11" t="s">
+      <c r="Q12" s="5" t="s">
         <v>393</v>
       </c>
-      <c r="R12" s="10" t="s">
+      <c r="R12" s="4" t="s">
         <v>394</v>
       </c>
-      <c r="S12" s="10" t="s">
+      <c r="S12" s="4" t="s">
         <v>392</v>
       </c>
-      <c r="T12" s="11" t="s">
+      <c r="T12" s="5" t="s">
         <v>393</v>
       </c>
       <c r="U12" t="b">
         <v>1</v>
       </c>
-      <c r="V12" s="12" t="s">
+      <c r="V12" s="7" t="s">
         <v>478</v>
       </c>
-    </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="W12" t="s">
+        <v>611</v>
+      </c>
+      <c r="X12" t="s">
+        <v>610</v>
+      </c>
+    </row>
+    <row r="13" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>25</v>
       </c>
@@ -3174,13 +3321,13 @@
         <f t="shared" si="0"/>
         <v>RothC results for year 2030 for Sorghum_rf_roff in ton C/ha</v>
       </c>
-      <c r="H13" s="10" t="s">
+      <c r="H13" s="4" t="s">
         <v>600</v>
       </c>
-      <c r="I13" s="10" t="s">
+      <c r="I13" s="4" t="s">
         <v>601</v>
       </c>
-      <c r="J13" s="11" t="s">
+      <c r="J13" s="5" t="s">
         <v>603</v>
       </c>
       <c r="N13" t="b">
@@ -3192,26 +3339,32 @@
       <c r="P13">
         <v>100</v>
       </c>
-      <c r="Q13" s="11" t="s">
+      <c r="Q13" s="5" t="s">
         <v>393</v>
       </c>
-      <c r="R13" s="10" t="s">
+      <c r="R13" s="4" t="s">
         <v>394</v>
       </c>
-      <c r="S13" s="10" t="s">
+      <c r="S13" s="4" t="s">
         <v>392</v>
       </c>
-      <c r="T13" s="11" t="s">
+      <c r="T13" s="5" t="s">
         <v>393</v>
       </c>
       <c r="U13" t="b">
         <v>1</v>
       </c>
-      <c r="V13" s="12" t="s">
+      <c r="V13" s="7" t="s">
         <v>478</v>
       </c>
-    </row>
-    <row r="14" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="W13" t="s">
+        <v>611</v>
+      </c>
+      <c r="X13" t="s">
+        <v>610</v>
+      </c>
+    </row>
+    <row r="14" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>26</v>
       </c>
@@ -3252,16 +3405,16 @@
       <c r="P14">
         <v>100</v>
       </c>
-      <c r="Q14" s="8" t="s">
+      <c r="Q14" s="6" t="s">
         <v>390</v>
       </c>
-      <c r="R14" s="7" t="s">
+      <c r="R14" s="3" t="s">
         <v>391</v>
       </c>
-      <c r="S14" s="7" t="s">
+      <c r="S14" s="3" t="s">
         <v>389</v>
       </c>
-      <c r="T14" s="8" t="s">
+      <c r="T14" s="6" t="s">
         <v>390</v>
       </c>
       <c r="U14" t="b">
@@ -3270,8 +3423,14 @@
       <c r="V14" t="s">
         <v>478</v>
       </c>
-    </row>
-    <row r="15" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="W14" t="s">
+        <v>611</v>
+      </c>
+      <c r="X14" t="s">
+        <v>610</v>
+      </c>
+    </row>
+    <row r="15" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>27</v>
       </c>
@@ -3297,10 +3456,10 @@
       <c r="H15" t="s">
         <v>608</v>
       </c>
-      <c r="I15" s="10" t="s">
+      <c r="I15" s="4" t="s">
         <v>546</v>
       </c>
-      <c r="J15" s="11" t="s">
+      <c r="J15" s="5" t="s">
         <v>548</v>
       </c>
       <c r="N15" t="b">
@@ -3312,16 +3471,16 @@
       <c r="P15">
         <v>100</v>
       </c>
-      <c r="Q15" s="8" t="s">
+      <c r="Q15" s="6" t="s">
         <v>396</v>
       </c>
-      <c r="R15" s="7" t="s">
+      <c r="R15" s="3" t="s">
         <v>397</v>
       </c>
-      <c r="S15" s="7" t="s">
+      <c r="S15" s="3" t="s">
         <v>395</v>
       </c>
-      <c r="T15" s="8" t="s">
+      <c r="T15" s="6" t="s">
         <v>396</v>
       </c>
       <c r="U15" t="b">
@@ -3330,8 +3489,14 @@
       <c r="V15" t="s">
         <v>478</v>
       </c>
-    </row>
-    <row r="16" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="W15" t="s">
+        <v>611</v>
+      </c>
+      <c r="X15" t="s">
+        <v>610</v>
+      </c>
+    </row>
+    <row r="16" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>29</v>
       </c>
@@ -3354,13 +3519,13 @@
         <f t="shared" si="0"/>
         <v>RothC results for year 2030 for Sunflower_rf in ton C/ha</v>
       </c>
-      <c r="H16" s="10" t="s">
+      <c r="H16" s="4" t="s">
         <v>569</v>
       </c>
-      <c r="I16" s="10" t="s">
+      <c r="I16" s="4" t="s">
         <v>570</v>
       </c>
-      <c r="J16" s="11" t="s">
+      <c r="J16" s="5" t="s">
         <v>571</v>
       </c>
       <c r="N16" t="b">
@@ -3372,16 +3537,16 @@
       <c r="P16">
         <v>100</v>
       </c>
-      <c r="Q16" s="11" t="s">
+      <c r="Q16" s="5" t="s">
         <v>387</v>
       </c>
-      <c r="R16" s="10" t="s">
+      <c r="R16" s="4" t="s">
         <v>388</v>
       </c>
-      <c r="S16" s="10" t="s">
+      <c r="S16" s="4" t="s">
         <v>386</v>
       </c>
-      <c r="T16" s="11" t="s">
+      <c r="T16" s="5" t="s">
         <v>387</v>
       </c>
       <c r="U16" t="b">
@@ -3390,8 +3555,14 @@
       <c r="V16" t="s">
         <v>478</v>
       </c>
-    </row>
-    <row r="17" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="W16" t="s">
+        <v>611</v>
+      </c>
+      <c r="X16" t="s">
+        <v>610</v>
+      </c>
+    </row>
+    <row r="17" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>30</v>
       </c>
@@ -3414,13 +3585,13 @@
         <f t="shared" si="0"/>
         <v>RothC results for year 2030 for Sweet potato_rf in ton C/ha</v>
       </c>
-      <c r="H17" s="7" t="s">
+      <c r="H17" s="3" t="s">
         <v>572</v>
       </c>
-      <c r="I17" s="7" t="s">
+      <c r="I17" s="3" t="s">
         <v>573</v>
       </c>
-      <c r="J17" s="8" t="s">
+      <c r="J17" s="6" t="s">
         <v>574</v>
       </c>
       <c r="N17" t="b">
@@ -3432,16 +3603,16 @@
       <c r="P17">
         <v>100</v>
       </c>
-      <c r="Q17" s="8" t="s">
+      <c r="Q17" s="6" t="s">
         <v>451</v>
       </c>
-      <c r="R17" s="7" t="s">
+      <c r="R17" s="3" t="s">
         <v>452</v>
       </c>
-      <c r="S17" s="7" t="s">
+      <c r="S17" s="3" t="s">
         <v>450</v>
       </c>
-      <c r="T17" s="8" t="s">
+      <c r="T17" s="6" t="s">
         <v>451</v>
       </c>
       <c r="U17" t="b">
@@ -3450,8 +3621,14 @@
       <c r="V17" t="s">
         <v>478</v>
       </c>
-    </row>
-    <row r="18" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="W17" t="s">
+        <v>611</v>
+      </c>
+      <c r="X17" t="s">
+        <v>610</v>
+      </c>
+    </row>
+    <row r="18" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>31</v>
       </c>
@@ -3474,13 +3651,13 @@
         <f t="shared" si="0"/>
         <v>RothC results for year 2030 for Tobacco_rf in ton C/ha</v>
       </c>
-      <c r="H18" s="10" t="s">
+      <c r="H18" s="4" t="s">
         <v>575</v>
       </c>
-      <c r="I18" s="10" t="s">
+      <c r="I18" s="4" t="s">
         <v>576</v>
       </c>
-      <c r="J18" s="11" t="s">
+      <c r="J18" s="5" t="s">
         <v>577</v>
       </c>
       <c r="N18" t="b">
@@ -3492,16 +3669,16 @@
       <c r="P18">
         <v>100</v>
       </c>
-      <c r="Q18" s="11" t="s">
+      <c r="Q18" s="5" t="s">
         <v>405</v>
       </c>
-      <c r="R18" s="10" t="s">
+      <c r="R18" s="4" t="s">
         <v>406</v>
       </c>
-      <c r="S18" s="10" t="s">
+      <c r="S18" s="4" t="s">
         <v>404</v>
       </c>
-      <c r="T18" s="11" t="s">
+      <c r="T18" s="5" t="s">
         <v>405</v>
       </c>
       <c r="U18" t="b">
@@ -3510,8 +3687,14 @@
       <c r="V18" t="s">
         <v>478</v>
       </c>
-    </row>
-    <row r="19" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="W18" t="s">
+        <v>611</v>
+      </c>
+      <c r="X18" t="s">
+        <v>610</v>
+      </c>
+    </row>
+    <row r="19" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>32</v>
       </c>
@@ -3534,13 +3717,13 @@
         <f t="shared" si="0"/>
         <v>RothC results for year 2030 for Tomato_rf in ton C/ha</v>
       </c>
-      <c r="H19" s="10" t="s">
+      <c r="H19" s="4" t="s">
         <v>578</v>
       </c>
-      <c r="I19" s="10" t="s">
+      <c r="I19" s="4" t="s">
         <v>562</v>
       </c>
-      <c r="J19" s="11" t="s">
+      <c r="J19" s="5" t="s">
         <v>564</v>
       </c>
       <c r="N19" t="b">
@@ -3552,16 +3735,16 @@
       <c r="P19">
         <v>100</v>
       </c>
-      <c r="Q19" s="8" t="s">
+      <c r="Q19" s="6" t="s">
         <v>408</v>
       </c>
-      <c r="R19" s="7" t="s">
+      <c r="R19" s="3" t="s">
         <v>409</v>
       </c>
-      <c r="S19" s="7" t="s">
+      <c r="S19" s="3" t="s">
         <v>407</v>
       </c>
-      <c r="T19" s="8" t="s">
+      <c r="T19" s="6" t="s">
         <v>408</v>
       </c>
       <c r="U19" t="b">
@@ -3570,8 +3753,14 @@
       <c r="V19" t="s">
         <v>478</v>
       </c>
-    </row>
-    <row r="20" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="W19" t="s">
+        <v>611</v>
+      </c>
+      <c r="X19" t="s">
+        <v>610</v>
+      </c>
+    </row>
+    <row r="20" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>33</v>
       </c>
@@ -3594,13 +3783,13 @@
         <f t="shared" si="0"/>
         <v>RothC results for year 2030 for Wheat_rf_ron in ton C/ha</v>
       </c>
-      <c r="H20" s="10" t="s">
+      <c r="H20" s="4" t="s">
         <v>581</v>
       </c>
-      <c r="I20" s="10" t="s">
+      <c r="I20" s="4" t="s">
         <v>582</v>
       </c>
-      <c r="J20" s="11" t="s">
+      <c r="J20" s="5" t="s">
         <v>583</v>
       </c>
       <c r="N20" t="b">
@@ -3612,16 +3801,16 @@
       <c r="P20">
         <v>100</v>
       </c>
-      <c r="Q20" s="11" t="s">
+      <c r="Q20" s="5" t="s">
         <v>411</v>
       </c>
-      <c r="R20" s="10" t="s">
+      <c r="R20" s="4" t="s">
         <v>412</v>
       </c>
-      <c r="S20" s="10" t="s">
+      <c r="S20" s="4" t="s">
         <v>410</v>
       </c>
-      <c r="T20" s="11" t="s">
+      <c r="T20" s="5" t="s">
         <v>411</v>
       </c>
       <c r="U20" t="b">
@@ -3630,8 +3819,14 @@
       <c r="V20" t="s">
         <v>478</v>
       </c>
-    </row>
-    <row r="21" spans="1:22" x14ac:dyDescent="0.35">
+      <c r="W20" t="s">
+        <v>611</v>
+      </c>
+      <c r="X20" t="s">
+        <v>610</v>
+      </c>
+    </row>
+    <row r="21" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>33</v>
       </c>
@@ -3654,13 +3849,13 @@
         <f t="shared" si="0"/>
         <v>RothC results for year 2030 for Wheat_rf_roff in ton C/ha</v>
       </c>
-      <c r="H21" s="10" t="s">
+      <c r="H21" s="4" t="s">
         <v>581</v>
       </c>
-      <c r="I21" s="10" t="s">
+      <c r="I21" s="4" t="s">
         <v>582</v>
       </c>
-      <c r="J21" s="11" t="s">
+      <c r="J21" s="5" t="s">
         <v>583</v>
       </c>
       <c r="N21" t="b">
@@ -3672,16 +3867,16 @@
       <c r="P21">
         <v>100</v>
       </c>
-      <c r="Q21" s="11" t="s">
+      <c r="Q21" s="5" t="s">
         <v>411</v>
       </c>
-      <c r="R21" s="10" t="s">
+      <c r="R21" s="4" t="s">
         <v>412</v>
       </c>
-      <c r="S21" s="10" t="s">
+      <c r="S21" s="4" t="s">
         <v>410</v>
       </c>
-      <c r="T21" s="11" t="s">
+      <c r="T21" s="5" t="s">
         <v>411</v>
       </c>
       <c r="U21" t="b">
@@ -3689,6 +3884,12 @@
       </c>
       <c r="V21" t="s">
         <v>478</v>
+      </c>
+      <c r="W21" t="s">
+        <v>611</v>
+      </c>
+      <c r="X21" t="s">
+        <v>610</v>
       </c>
     </row>
   </sheetData>
@@ -3733,784 +3934,784 @@
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A2" s="6" t="s">
+      <c r="A2" t="s">
         <v>15</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" t="s">
         <v>503</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" t="s">
         <v>504</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" t="s">
         <v>335</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" t="s">
         <v>505</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="F2" t="s">
         <v>506</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="G2" t="s">
         <v>507</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A3" s="6" t="s">
+      <c r="A3" t="s">
         <v>16</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" t="s">
         <v>503</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" t="s">
         <v>508</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" t="s">
         <v>509</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="E3" t="s">
         <v>510</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="F3" t="s">
         <v>511</v>
       </c>
-      <c r="G3" s="6" t="s">
+      <c r="G3" t="s">
         <v>512</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A4" s="6" t="s">
+      <c r="A4" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" t="s">
         <v>503</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" t="s">
         <v>508</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D4" t="s">
         <v>513</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="E4" t="s">
         <v>514</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="F4" t="s">
         <v>515</v>
       </c>
-      <c r="G4" s="6" t="s">
+      <c r="G4" t="s">
         <v>516</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A5" s="6" t="s">
+      <c r="A5" t="s">
         <v>18</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" t="s">
         <v>503</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" t="s">
         <v>508</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" t="s">
         <v>517</v>
       </c>
-      <c r="E5" s="6" t="s">
+      <c r="E5" t="s">
         <v>518</v>
       </c>
-      <c r="F5" s="6" t="s">
+      <c r="F5" t="s">
         <v>519</v>
       </c>
-      <c r="G5" s="6" t="s">
+      <c r="G5" t="s">
         <v>520</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A6" s="6" t="s">
+      <c r="A6" t="s">
         <v>20</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" t="s">
         <v>503</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" t="s">
         <v>504</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="D6" t="s">
         <v>521</v>
       </c>
-      <c r="E6" s="6" t="s">
+      <c r="E6" t="s">
         <v>522</v>
       </c>
-      <c r="F6" s="6" t="s">
+      <c r="F6" t="s">
         <v>523</v>
       </c>
-      <c r="G6" s="6" t="s">
+      <c r="G6" t="s">
         <v>524</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A7" s="6" t="s">
+      <c r="A7" t="s">
         <v>21</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" t="s">
         <v>503</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" t="s">
         <v>508</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="D7" t="s">
         <v>525</v>
       </c>
-      <c r="E7" s="6" t="s">
+      <c r="E7" t="s">
         <v>526</v>
       </c>
-      <c r="F7" s="6" t="s">
+      <c r="F7" t="s">
         <v>527</v>
       </c>
-      <c r="G7" s="6" t="s">
+      <c r="G7" t="s">
         <v>528</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A8" s="6" t="s">
+      <c r="A8" t="s">
         <v>22</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B8" t="s">
         <v>503</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="C8" t="s">
         <v>508</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="D8" t="s">
         <v>529</v>
       </c>
-      <c r="E8" s="6" t="s">
+      <c r="E8" t="s">
         <v>530</v>
       </c>
-      <c r="F8" s="6" t="s">
+      <c r="F8" t="s">
         <v>531</v>
       </c>
-      <c r="G8" s="6" t="s">
+      <c r="G8" t="s">
         <v>532</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A9" s="6" t="s">
+      <c r="A9" t="s">
         <v>23</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" t="s">
         <v>503</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="C9" t="s">
         <v>504</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="D9" t="s">
         <v>533</v>
       </c>
-      <c r="E9" s="6" t="s">
+      <c r="E9" t="s">
         <v>534</v>
       </c>
-      <c r="F9" s="6" t="s">
+      <c r="F9" t="s">
         <v>535</v>
       </c>
-      <c r="G9" s="6" t="s">
+      <c r="G9" t="s">
         <v>536</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A10" s="6" t="s">
+      <c r="A10" t="s">
         <v>25</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="B10" t="s">
         <v>503</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="C10" t="s">
         <v>504</v>
       </c>
-      <c r="D10" s="6" t="s">
+      <c r="D10" t="s">
         <v>537</v>
       </c>
-      <c r="E10" s="6" t="s">
+      <c r="E10" t="s">
         <v>538</v>
       </c>
-      <c r="F10" s="6" t="s">
+      <c r="F10" t="s">
         <v>539</v>
       </c>
-      <c r="G10" s="6" t="s">
+      <c r="G10" t="s">
         <v>540</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A11" s="6" t="s">
+      <c r="A11" t="s">
         <v>26</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="B11" t="s">
         <v>503</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="C11" t="s">
         <v>508</v>
       </c>
-      <c r="D11" s="6" t="s">
+      <c r="D11" t="s">
         <v>541</v>
       </c>
-      <c r="E11" s="6" t="s">
+      <c r="E11" t="s">
         <v>542</v>
       </c>
-      <c r="F11" s="6" t="s">
+      <c r="F11" t="s">
         <v>543</v>
       </c>
-      <c r="G11" s="6" t="s">
+      <c r="G11" t="s">
         <v>544</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A12" s="6" t="s">
+      <c r="A12" t="s">
         <v>27</v>
       </c>
-      <c r="B12" s="6" t="s">
+      <c r="B12" t="s">
         <v>503</v>
       </c>
-      <c r="C12" s="6" t="s">
+      <c r="C12" t="s">
         <v>508</v>
       </c>
-      <c r="D12" s="6" t="s">
+      <c r="D12" t="s">
         <v>545</v>
       </c>
-      <c r="E12" s="6" t="s">
+      <c r="E12" t="s">
         <v>546</v>
       </c>
-      <c r="F12" s="6" t="s">
+      <c r="F12" t="s">
         <v>547</v>
       </c>
-      <c r="G12" s="6" t="s">
+      <c r="G12" t="s">
         <v>548</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A13" s="6" t="s">
+      <c r="A13" t="s">
         <v>29</v>
       </c>
-      <c r="B13" s="6" t="s">
+      <c r="B13" t="s">
         <v>503</v>
       </c>
-      <c r="C13" s="6" t="s">
+      <c r="C13" t="s">
         <v>508</v>
       </c>
-      <c r="D13" s="6" t="s">
+      <c r="D13" t="s">
         <v>549</v>
       </c>
-      <c r="E13" s="6" t="s">
+      <c r="E13" t="s">
         <v>550</v>
       </c>
-      <c r="F13" s="6" t="s">
+      <c r="F13" t="s">
         <v>551</v>
       </c>
-      <c r="G13" s="6" t="s">
+      <c r="G13" t="s">
         <v>552</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A14" s="6" t="s">
+      <c r="A14" t="s">
         <v>30</v>
       </c>
-      <c r="B14" s="6" t="s">
+      <c r="B14" t="s">
         <v>503</v>
       </c>
-      <c r="C14" s="6" t="s">
+      <c r="C14" t="s">
         <v>508</v>
       </c>
-      <c r="D14" s="6" t="s">
+      <c r="D14" t="s">
         <v>553</v>
       </c>
-      <c r="E14" s="6" t="s">
+      <c r="E14" t="s">
         <v>554</v>
       </c>
-      <c r="F14" s="6" t="s">
+      <c r="F14" t="s">
         <v>555</v>
       </c>
-      <c r="G14" s="6" t="s">
+      <c r="G14" t="s">
         <v>556</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A15" s="6" t="s">
+      <c r="A15" t="s">
         <v>31</v>
       </c>
-      <c r="B15" s="6" t="s">
+      <c r="B15" t="s">
         <v>503</v>
       </c>
-      <c r="C15" s="6" t="s">
+      <c r="C15" t="s">
         <v>508</v>
       </c>
-      <c r="D15" s="6" t="s">
+      <c r="D15" t="s">
         <v>557</v>
       </c>
-      <c r="E15" s="6" t="s">
+      <c r="E15" t="s">
         <v>558</v>
       </c>
-      <c r="F15" s="6" t="s">
+      <c r="F15" t="s">
         <v>559</v>
       </c>
-      <c r="G15" s="6" t="s">
+      <c r="G15" t="s">
         <v>560</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A16" s="6" t="s">
+      <c r="A16" t="s">
         <v>32</v>
       </c>
-      <c r="B16" s="6" t="s">
+      <c r="B16" t="s">
         <v>503</v>
       </c>
-      <c r="C16" s="6" t="s">
+      <c r="C16" t="s">
         <v>508</v>
       </c>
-      <c r="D16" s="6" t="s">
+      <c r="D16" t="s">
         <v>561</v>
       </c>
-      <c r="E16" s="6" t="s">
+      <c r="E16" t="s">
         <v>562</v>
       </c>
-      <c r="F16" s="6" t="s">
+      <c r="F16" t="s">
         <v>563</v>
       </c>
-      <c r="G16" s="6" t="s">
+      <c r="G16" t="s">
         <v>564</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A17" s="6" t="s">
+      <c r="A17" t="s">
         <v>33</v>
       </c>
-      <c r="B17" s="6" t="s">
+      <c r="B17" t="s">
         <v>503</v>
       </c>
-      <c r="C17" s="6" t="s">
+      <c r="C17" t="s">
         <v>504</v>
       </c>
-      <c r="D17" s="6" t="s">
+      <c r="D17" t="s">
         <v>565</v>
       </c>
-      <c r="E17" s="6" t="s">
+      <c r="E17" t="s">
         <v>566</v>
       </c>
-      <c r="F17" s="6" t="s">
+      <c r="F17" t="s">
         <v>567</v>
       </c>
-      <c r="G17" s="6" t="s">
+      <c r="G17" t="s">
         <v>568</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A18" s="6" t="s">
+      <c r="A18" t="s">
         <v>15</v>
       </c>
-      <c r="B18" s="6" t="s">
+      <c r="B18" t="s">
         <v>503</v>
       </c>
-      <c r="C18" s="6" t="s">
+      <c r="C18" t="s">
         <v>35</v>
       </c>
-      <c r="D18" s="6" t="s">
+      <c r="D18" t="s">
         <v>336</v>
       </c>
-      <c r="E18" s="6" t="s">
+      <c r="E18" t="s">
         <v>337</v>
       </c>
-      <c r="F18" s="6" t="s">
+      <c r="F18" t="s">
         <v>346</v>
       </c>
-      <c r="G18" s="6" t="s">
+      <c r="G18" t="s">
         <v>338</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A19" s="6" t="s">
+      <c r="A19" t="s">
         <v>18</v>
       </c>
-      <c r="B19" s="6" t="s">
+      <c r="B19" t="s">
         <v>503</v>
       </c>
-      <c r="C19" s="6" t="s">
+      <c r="C19" t="s">
         <v>37</v>
       </c>
-      <c r="D19" s="6" t="s">
+      <c r="D19" t="s">
         <v>479</v>
       </c>
-      <c r="E19" s="6" t="s">
+      <c r="E19" t="s">
         <v>480</v>
       </c>
-      <c r="F19" s="6" t="s">
+      <c r="F19" t="s">
         <v>346</v>
       </c>
-      <c r="G19" s="6" t="s">
+      <c r="G19" t="s">
         <v>481</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A20" s="6" t="s">
+      <c r="A20" t="s">
         <v>20</v>
       </c>
-      <c r="B20" s="6" t="s">
+      <c r="B20" t="s">
         <v>503</v>
       </c>
-      <c r="C20" s="6" t="s">
+      <c r="C20" t="s">
         <v>35</v>
       </c>
-      <c r="D20" s="6" t="s">
+      <c r="D20" t="s">
         <v>485</v>
       </c>
-      <c r="E20" s="6" t="s">
+      <c r="E20" t="s">
         <v>486</v>
       </c>
-      <c r="F20" s="6" t="s">
+      <c r="F20" t="s">
         <v>346</v>
       </c>
-      <c r="G20" s="6" t="s">
+      <c r="G20" t="s">
         <v>487</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A21" s="6" t="s">
+      <c r="A21" t="s">
         <v>22</v>
       </c>
-      <c r="B21" s="6" t="s">
+      <c r="B21" t="s">
         <v>503</v>
       </c>
-      <c r="C21" s="6" t="s">
+      <c r="C21" t="s">
         <v>37</v>
       </c>
-      <c r="D21" s="6" t="s">
+      <c r="D21" t="s">
         <v>488</v>
       </c>
-      <c r="E21" s="6" t="s">
+      <c r="E21" t="s">
         <v>489</v>
       </c>
-      <c r="F21" s="6" t="s">
+      <c r="F21" t="s">
         <v>346</v>
       </c>
-      <c r="G21" s="6" t="s">
+      <c r="G21" t="s">
         <v>490</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A22" s="6" t="s">
+      <c r="A22" t="s">
         <v>23</v>
       </c>
-      <c r="B22" s="6" t="s">
+      <c r="B22" t="s">
         <v>503</v>
       </c>
-      <c r="C22" s="6" t="s">
+      <c r="C22" t="s">
         <v>35</v>
       </c>
-      <c r="D22" s="6" t="s">
+      <c r="D22" t="s">
         <v>491</v>
       </c>
-      <c r="E22" s="6" t="s">
+      <c r="E22" t="s">
         <v>492</v>
       </c>
-      <c r="F22" s="6" t="s">
+      <c r="F22" t="s">
         <v>346</v>
       </c>
-      <c r="G22" s="6" t="s">
+      <c r="G22" t="s">
         <v>493</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A23" s="6" t="s">
+      <c r="A23" t="s">
         <v>26</v>
       </c>
-      <c r="B23" s="6" t="s">
+      <c r="B23" t="s">
         <v>503</v>
       </c>
-      <c r="C23" s="6" t="s">
+      <c r="C23" t="s">
         <v>37</v>
       </c>
-      <c r="D23" s="6" t="s">
+      <c r="D23" t="s">
         <v>494</v>
       </c>
-      <c r="E23" s="6" t="s">
+      <c r="E23" t="s">
         <v>495</v>
       </c>
-      <c r="F23" s="6" t="s">
+      <c r="F23" t="s">
         <v>346</v>
       </c>
-      <c r="G23" s="6" t="s">
+      <c r="G23" t="s">
         <v>496</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A24" s="6" t="s">
+      <c r="A24" t="s">
         <v>29</v>
       </c>
-      <c r="B24" s="6" t="s">
+      <c r="B24" t="s">
         <v>503</v>
       </c>
-      <c r="C24" s="6" t="s">
+      <c r="C24" t="s">
         <v>37</v>
       </c>
-      <c r="D24" s="6" t="s">
+      <c r="D24" t="s">
         <v>569</v>
       </c>
-      <c r="E24" s="6" t="s">
+      <c r="E24" t="s">
         <v>570</v>
       </c>
-      <c r="F24" s="6" t="s">
+      <c r="F24" t="s">
         <v>346</v>
       </c>
-      <c r="G24" s="6" t="s">
+      <c r="G24" t="s">
         <v>571</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A25" s="6" t="s">
+      <c r="A25" t="s">
         <v>30</v>
       </c>
-      <c r="B25" s="6" t="s">
+      <c r="B25" t="s">
         <v>503</v>
       </c>
-      <c r="C25" s="6" t="s">
+      <c r="C25" t="s">
         <v>37</v>
       </c>
-      <c r="D25" s="6" t="s">
+      <c r="D25" t="s">
         <v>572</v>
       </c>
-      <c r="E25" s="6" t="s">
+      <c r="E25" t="s">
         <v>573</v>
       </c>
-      <c r="F25" s="6" t="s">
+      <c r="F25" t="s">
         <v>346</v>
       </c>
-      <c r="G25" s="6" t="s">
+      <c r="G25" t="s">
         <v>574</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A26" s="6" t="s">
+      <c r="A26" t="s">
         <v>31</v>
       </c>
-      <c r="B26" s="6" t="s">
+      <c r="B26" t="s">
         <v>503</v>
       </c>
-      <c r="C26" s="6" t="s">
+      <c r="C26" t="s">
         <v>37</v>
       </c>
-      <c r="D26" s="6" t="s">
+      <c r="D26" t="s">
         <v>575</v>
       </c>
-      <c r="E26" s="6" t="s">
+      <c r="E26" t="s">
         <v>576</v>
       </c>
-      <c r="F26" s="6" t="s">
+      <c r="F26" t="s">
         <v>346</v>
       </c>
-      <c r="G26" s="6" t="s">
+      <c r="G26" t="s">
         <v>577</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A27" s="6" t="s">
+      <c r="A27" t="s">
         <v>32</v>
       </c>
-      <c r="B27" s="6" t="s">
+      <c r="B27" t="s">
         <v>503</v>
       </c>
-      <c r="C27" s="6" t="s">
+      <c r="C27" t="s">
         <v>37</v>
       </c>
-      <c r="D27" s="6" t="s">
+      <c r="D27" t="s">
         <v>578</v>
       </c>
-      <c r="E27" s="6" t="s">
+      <c r="E27" t="s">
         <v>579</v>
       </c>
-      <c r="F27" s="6" t="s">
+      <c r="F27" t="s">
         <v>346</v>
       </c>
-      <c r="G27" s="6" t="s">
+      <c r="G27" t="s">
         <v>580</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A28" s="6" t="s">
+      <c r="A28" t="s">
         <v>33</v>
       </c>
-      <c r="B28" s="6" t="s">
+      <c r="B28" t="s">
         <v>503</v>
       </c>
-      <c r="C28" s="6" t="s">
+      <c r="C28" t="s">
         <v>35</v>
       </c>
-      <c r="D28" s="6" t="s">
+      <c r="D28" t="s">
         <v>581</v>
       </c>
-      <c r="E28" s="6" t="s">
+      <c r="E28" t="s">
         <v>582</v>
       </c>
-      <c r="F28" s="6" t="s">
+      <c r="F28" t="s">
         <v>346</v>
       </c>
-      <c r="G28" s="6" t="s">
+      <c r="G28" t="s">
         <v>583</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A29" s="6" t="s">
+      <c r="A29" t="s">
         <v>19</v>
       </c>
-      <c r="B29" s="6" t="s">
+      <c r="B29" t="s">
         <v>503</v>
       </c>
-      <c r="C29" s="6" t="s">
+      <c r="C29" t="s">
         <v>508</v>
       </c>
-      <c r="D29" s="6" t="s">
+      <c r="D29" t="s">
         <v>584</v>
       </c>
-      <c r="E29" s="6" t="s">
+      <c r="E29" t="s">
         <v>585</v>
       </c>
-      <c r="F29" s="6" t="s">
+      <c r="F29" t="s">
         <v>586</v>
       </c>
-      <c r="G29" s="6" t="s">
+      <c r="G29" t="s">
         <v>587</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A30" s="6" t="s">
+      <c r="A30" t="s">
         <v>19</v>
       </c>
-      <c r="B30" s="6" t="s">
+      <c r="B30" t="s">
         <v>503</v>
       </c>
-      <c r="C30" s="6" t="s">
+      <c r="C30" t="s">
         <v>37</v>
       </c>
-      <c r="D30" s="6" t="s">
+      <c r="D30" t="s">
         <v>482</v>
       </c>
-      <c r="E30" s="6" t="s">
+      <c r="E30" t="s">
         <v>483</v>
       </c>
-      <c r="F30" s="6" t="s">
+      <c r="F30" t="s">
         <v>346</v>
       </c>
-      <c r="G30" s="6" t="s">
+      <c r="G30" t="s">
         <v>484</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A31" s="6" t="s">
+      <c r="A31" t="s">
         <v>15</v>
       </c>
-      <c r="B31" s="6" t="s">
+      <c r="B31" t="s">
         <v>503</v>
       </c>
-      <c r="C31" s="6" t="s">
+      <c r="C31" t="s">
         <v>588</v>
       </c>
-      <c r="D31" s="6" t="s">
+      <c r="D31" t="s">
         <v>589</v>
       </c>
-      <c r="E31" s="6" t="s">
+      <c r="E31" t="s">
         <v>590</v>
       </c>
-      <c r="F31" s="6" t="s">
+      <c r="F31" t="s">
         <v>591</v>
       </c>
-      <c r="G31" s="6" t="s">
+      <c r="G31" t="s">
         <v>592</v>
       </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A32" s="6" t="s">
+      <c r="A32" t="s">
         <v>20</v>
       </c>
-      <c r="B32" s="6" t="s">
+      <c r="B32" t="s">
         <v>503</v>
       </c>
-      <c r="C32" s="6" t="s">
+      <c r="C32" t="s">
         <v>588</v>
       </c>
-      <c r="D32" s="6" t="s">
+      <c r="D32" t="s">
         <v>593</v>
       </c>
-      <c r="E32" s="6" t="s">
+      <c r="E32" t="s">
         <v>594</v>
       </c>
-      <c r="F32" s="6" t="s">
+      <c r="F32" t="s">
         <v>595</v>
       </c>
-      <c r="G32" s="6" t="s">
+      <c r="G32" t="s">
         <v>596</v>
       </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A33" s="6" t="s">
+      <c r="A33" t="s">
         <v>23</v>
       </c>
-      <c r="B33" s="6" t="s">
+      <c r="B33" t="s">
         <v>503</v>
       </c>
-      <c r="C33" s="6" t="s">
+      <c r="C33" t="s">
         <v>588</v>
       </c>
-      <c r="D33" s="6" t="s">
+      <c r="D33" t="s">
         <v>533</v>
       </c>
-      <c r="E33" s="6" t="s">
+      <c r="E33" t="s">
         <v>597</v>
       </c>
-      <c r="F33" s="6" t="s">
+      <c r="F33" t="s">
         <v>598</v>
       </c>
-      <c r="G33" s="6" t="s">
+      <c r="G33" t="s">
         <v>599</v>
       </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A34" s="6" t="s">
+      <c r="A34" t="s">
         <v>25</v>
       </c>
-      <c r="B34" s="6" t="s">
+      <c r="B34" t="s">
         <v>503</v>
       </c>
-      <c r="C34" s="6" t="s">
+      <c r="C34" t="s">
         <v>588</v>
       </c>
-      <c r="D34" s="6" t="s">
+      <c r="D34" t="s">
         <v>600</v>
       </c>
-      <c r="E34" s="6" t="s">
+      <c r="E34" t="s">
         <v>601</v>
       </c>
-      <c r="F34" s="6" t="s">
+      <c r="F34" t="s">
         <v>602</v>
       </c>
-      <c r="G34" s="6" t="s">
+      <c r="G34" t="s">
         <v>603</v>
       </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A35" s="6" t="s">
+      <c r="A35" t="s">
         <v>33</v>
       </c>
-      <c r="B35" s="6" t="s">
+      <c r="B35" t="s">
         <v>503</v>
       </c>
-      <c r="C35" s="6" t="s">
+      <c r="C35" t="s">
         <v>588</v>
       </c>
-      <c r="D35" s="6" t="s">
+      <c r="D35" t="s">
         <v>604</v>
       </c>
-      <c r="E35" s="6" t="s">
+      <c r="E35" t="s">
         <v>605</v>
       </c>
-      <c r="F35" s="6" t="s">
+      <c r="F35" t="s">
         <v>606</v>
       </c>
-      <c r="G35" s="6" t="s">
+      <c r="G35" t="s">
         <v>607</v>
       </c>
     </row>
@@ -4548,520 +4749,520 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="6" t="s">
+      <c r="A2" t="s">
         <v>413</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" t="s">
         <v>342</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" t="s">
         <v>340</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" t="s">
         <v>341</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" s="6" t="s">
+      <c r="A3" t="s">
         <v>15</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" t="s">
         <v>345</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" t="s">
         <v>343</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" t="s">
         <v>344</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A4" s="6" t="s">
+      <c r="A4" t="s">
         <v>414</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" t="s">
         <v>349</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" t="s">
         <v>347</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D4" t="s">
         <v>348</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A5" s="6" t="s">
+      <c r="A5" t="s">
         <v>59</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" t="s">
         <v>352</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" t="s">
         <v>350</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" t="s">
         <v>351</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6" s="6" t="s">
+      <c r="A6" t="s">
         <v>65</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" t="s">
         <v>355</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" t="s">
         <v>353</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="D6" t="s">
         <v>354</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A7" s="6" t="s">
+      <c r="A7" t="s">
         <v>62</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" t="s">
         <v>358</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" t="s">
         <v>356</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="D7" t="s">
         <v>357</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A8" s="6" t="s">
+      <c r="A8" t="s">
         <v>415</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B8" t="s">
         <v>361</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="C8" t="s">
         <v>359</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="D8" t="s">
         <v>360</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A9" s="6" t="s">
+      <c r="A9" t="s">
         <v>142</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" t="s">
         <v>364</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="C9" t="s">
         <v>362</v>
       </c>
-      <c r="D9" s="6" t="s">
+      <c r="D9" t="s">
         <v>363</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A10" s="6" t="s">
+      <c r="A10" t="s">
         <v>416</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="B10" t="s">
         <v>419</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="C10" t="s">
         <v>417</v>
       </c>
-      <c r="D10" s="6" t="s">
+      <c r="D10" t="s">
         <v>418</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A11" s="6" t="s">
+      <c r="A11" t="s">
         <v>420</v>
       </c>
-      <c r="B11" s="6" t="s">
+      <c r="B11" t="s">
         <v>423</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="C11" t="s">
         <v>421</v>
       </c>
-      <c r="D11" s="6" t="s">
+      <c r="D11" t="s">
         <v>422</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A12" s="6" t="s">
+      <c r="A12" t="s">
         <v>424</v>
       </c>
-      <c r="B12" s="6" t="s">
+      <c r="B12" t="s">
         <v>367</v>
       </c>
-      <c r="C12" s="6" t="s">
+      <c r="C12" t="s">
         <v>365</v>
       </c>
-      <c r="D12" s="6" t="s">
+      <c r="D12" t="s">
         <v>366</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A13" s="6" t="s">
+      <c r="A13" t="s">
         <v>425</v>
       </c>
-      <c r="B13" s="6" t="s">
+      <c r="B13" t="s">
         <v>428</v>
       </c>
-      <c r="C13" s="6" t="s">
+      <c r="C13" t="s">
         <v>426</v>
       </c>
-      <c r="D13" s="6" t="s">
+      <c r="D13" t="s">
         <v>427</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A14" s="6" t="s">
+      <c r="A14" t="s">
         <v>429</v>
       </c>
-      <c r="B14" s="6" t="s">
+      <c r="B14" t="s">
         <v>432</v>
       </c>
-      <c r="C14" s="6" t="s">
+      <c r="C14" t="s">
         <v>430</v>
       </c>
-      <c r="D14" s="6" t="s">
+      <c r="D14" t="s">
         <v>431</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A15" s="6" t="s">
+      <c r="A15" t="s">
         <v>20</v>
       </c>
-      <c r="B15" s="6" t="s">
+      <c r="B15" t="s">
         <v>370</v>
       </c>
-      <c r="C15" s="6" t="s">
+      <c r="C15" t="s">
         <v>368</v>
       </c>
-      <c r="D15" s="6" t="s">
+      <c r="D15" t="s">
         <v>369</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A16" s="6" t="s">
+      <c r="A16" t="s">
         <v>433</v>
       </c>
-      <c r="B16" s="6" t="s">
+      <c r="B16" t="s">
         <v>436</v>
       </c>
-      <c r="C16" s="6" t="s">
+      <c r="C16" t="s">
         <v>434</v>
       </c>
-      <c r="D16" s="6" t="s">
+      <c r="D16" t="s">
         <v>435</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A17" s="6" t="s">
+      <c r="A17" t="s">
         <v>437</v>
       </c>
-      <c r="B17" s="6" t="s">
+      <c r="B17" t="s">
         <v>440</v>
       </c>
-      <c r="C17" s="6" t="s">
+      <c r="C17" t="s">
         <v>438</v>
       </c>
-      <c r="D17" s="6" t="s">
+      <c r="D17" t="s">
         <v>439</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A18" s="6" t="s">
+      <c r="A18" t="s">
         <v>441</v>
       </c>
-      <c r="B18" s="6" t="s">
+      <c r="B18" t="s">
         <v>444</v>
       </c>
-      <c r="C18" s="6" t="s">
+      <c r="C18" t="s">
         <v>442</v>
       </c>
-      <c r="D18" s="6" t="s">
+      <c r="D18" t="s">
         <v>443</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A19" s="6" t="s">
+      <c r="A19" t="s">
         <v>78</v>
       </c>
-      <c r="B19" s="6" t="s">
+      <c r="B19" t="s">
         <v>373</v>
       </c>
-      <c r="C19" s="6" t="s">
+      <c r="C19" t="s">
         <v>371</v>
       </c>
-      <c r="D19" s="6" t="s">
+      <c r="D19" t="s">
         <v>372</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A20" s="6" t="s">
+      <c r="A20" t="s">
         <v>445</v>
       </c>
-      <c r="B20" s="6" t="s">
+      <c r="B20" t="s">
         <v>448</v>
       </c>
-      <c r="C20" s="6" t="s">
+      <c r="C20" t="s">
         <v>446</v>
       </c>
-      <c r="D20" s="6" t="s">
+      <c r="D20" t="s">
         <v>447</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A21" s="6" t="s">
+      <c r="A21" t="s">
         <v>449</v>
       </c>
-      <c r="B21" s="6" t="s">
+      <c r="B21" t="s">
         <v>452</v>
       </c>
-      <c r="C21" s="6" t="s">
+      <c r="C21" t="s">
         <v>450</v>
       </c>
-      <c r="D21" s="6" t="s">
+      <c r="D21" t="s">
         <v>451</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A22" s="6" t="s">
+      <c r="A22" t="s">
         <v>453</v>
       </c>
-      <c r="B22" s="6" t="s">
+      <c r="B22" t="s">
         <v>456</v>
       </c>
-      <c r="C22" s="6" t="s">
+      <c r="C22" t="s">
         <v>454</v>
       </c>
-      <c r="D22" s="6" t="s">
+      <c r="D22" t="s">
         <v>455</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A23" s="6" t="s">
+      <c r="A23" t="s">
         <v>457</v>
       </c>
-      <c r="B23" s="6" t="s">
+      <c r="B23" t="s">
         <v>460</v>
       </c>
-      <c r="C23" s="6" t="s">
+      <c r="C23" t="s">
         <v>458</v>
       </c>
-      <c r="D23" s="6" t="s">
+      <c r="D23" t="s">
         <v>459</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A24" s="6" t="s">
+      <c r="A24" t="s">
         <v>461</v>
       </c>
-      <c r="B24" s="6" t="s">
+      <c r="B24" t="s">
         <v>464</v>
       </c>
-      <c r="C24" s="6" t="s">
+      <c r="C24" t="s">
         <v>462</v>
       </c>
-      <c r="D24" s="6" t="s">
+      <c r="D24" t="s">
         <v>463</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A25" s="6" t="s">
+      <c r="A25" t="s">
         <v>24</v>
       </c>
-      <c r="B25" s="6" t="s">
+      <c r="B25" t="s">
         <v>376</v>
       </c>
-      <c r="C25" s="6" t="s">
+      <c r="C25" t="s">
         <v>374</v>
       </c>
-      <c r="D25" s="6" t="s">
+      <c r="D25" t="s">
         <v>375</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A26" s="6" t="s">
+      <c r="A26" t="s">
         <v>23</v>
       </c>
-      <c r="B26" s="6" t="s">
+      <c r="B26" t="s">
         <v>379</v>
       </c>
-      <c r="C26" s="6" t="s">
+      <c r="C26" t="s">
         <v>377</v>
       </c>
-      <c r="D26" s="6" t="s">
+      <c r="D26" t="s">
         <v>378</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A27" s="6" t="s">
+      <c r="A27" t="s">
         <v>465</v>
       </c>
-      <c r="B27" s="6" t="s">
+      <c r="B27" t="s">
         <v>468</v>
       </c>
-      <c r="C27" s="6" t="s">
+      <c r="C27" t="s">
         <v>466</v>
       </c>
-      <c r="D27" s="6" t="s">
+      <c r="D27" t="s">
         <v>467</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A28" s="6" t="s">
+      <c r="A28" t="s">
         <v>469</v>
       </c>
-      <c r="B28" s="6" t="s">
+      <c r="B28" t="s">
         <v>382</v>
       </c>
-      <c r="C28" s="6" t="s">
+      <c r="C28" t="s">
         <v>380</v>
       </c>
-      <c r="D28" s="6" t="s">
+      <c r="D28" t="s">
         <v>381</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A29" s="6" t="s">
+      <c r="A29" t="s">
         <v>470</v>
       </c>
-      <c r="B29" s="6" t="s">
+      <c r="B29" t="s">
         <v>385</v>
       </c>
-      <c r="C29" s="6" t="s">
+      <c r="C29" t="s">
         <v>383</v>
       </c>
-      <c r="D29" s="6" t="s">
+      <c r="D29" t="s">
         <v>384</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A30" s="6" t="s">
+      <c r="A30" t="s">
         <v>104</v>
       </c>
-      <c r="B30" s="6" t="s">
+      <c r="B30" t="s">
         <v>388</v>
       </c>
-      <c r="C30" s="6" t="s">
+      <c r="C30" t="s">
         <v>386</v>
       </c>
-      <c r="D30" s="6" t="s">
+      <c r="D30" t="s">
         <v>387</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A31" s="6" t="s">
+      <c r="A31" t="s">
         <v>26</v>
       </c>
-      <c r="B31" s="6" t="s">
+      <c r="B31" t="s">
         <v>391</v>
       </c>
-      <c r="C31" s="6" t="s">
+      <c r="C31" t="s">
         <v>389</v>
       </c>
-      <c r="D31" s="6" t="s">
+      <c r="D31" t="s">
         <v>390</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A32" s="6" t="s">
+      <c r="A32" t="s">
         <v>25</v>
       </c>
-      <c r="B32" s="6" t="s">
+      <c r="B32" t="s">
         <v>394</v>
       </c>
-      <c r="C32" s="6" t="s">
+      <c r="C32" t="s">
         <v>392</v>
       </c>
-      <c r="D32" s="6" t="s">
+      <c r="D32" t="s">
         <v>393</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A33" s="6" t="s">
+      <c r="A33" t="s">
         <v>27</v>
       </c>
-      <c r="B33" s="6" t="s">
+      <c r="B33" t="s">
         <v>397</v>
       </c>
-      <c r="C33" s="6" t="s">
+      <c r="C33" t="s">
         <v>395</v>
       </c>
-      <c r="D33" s="6" t="s">
+      <c r="D33" t="s">
         <v>396</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A34" s="6" t="s">
+      <c r="A34" t="s">
         <v>28</v>
       </c>
-      <c r="B34" s="6" t="s">
+      <c r="B34" t="s">
         <v>400</v>
       </c>
-      <c r="C34" s="6" t="s">
+      <c r="C34" t="s">
         <v>398</v>
       </c>
-      <c r="D34" s="6" t="s">
+      <c r="D34" t="s">
         <v>399</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A35" s="6" t="s">
+      <c r="A35" t="s">
         <v>471</v>
       </c>
-      <c r="B35" s="6" t="s">
+      <c r="B35" t="s">
         <v>403</v>
       </c>
-      <c r="C35" s="6" t="s">
+      <c r="C35" t="s">
         <v>401</v>
       </c>
-      <c r="D35" s="6" t="s">
+      <c r="D35" t="s">
         <v>402</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A36" s="6" t="s">
+      <c r="A36" t="s">
         <v>472</v>
       </c>
-      <c r="B36" s="6" t="s">
+      <c r="B36" t="s">
         <v>406</v>
       </c>
-      <c r="C36" s="6" t="s">
+      <c r="C36" t="s">
         <v>404</v>
       </c>
-      <c r="D36" s="6" t="s">
+      <c r="D36" t="s">
         <v>405</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A37" s="6" t="s">
+      <c r="A37" t="s">
         <v>32</v>
       </c>
-      <c r="B37" s="6" t="s">
+      <c r="B37" t="s">
         <v>409</v>
       </c>
-      <c r="C37" s="6" t="s">
+      <c r="C37" t="s">
         <v>407</v>
       </c>
-      <c r="D37" s="6" t="s">
+      <c r="D37" t="s">
         <v>408</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A38" s="6" t="s">
+      <c r="A38" t="s">
         <v>33</v>
       </c>
-      <c r="B38" s="6" t="s">
+      <c r="B38" t="s">
         <v>412</v>
       </c>
-      <c r="C38" s="6" t="s">
+      <c r="C38" t="s">
         <v>410</v>
       </c>
-      <c r="D38" s="6" t="s">
+      <c r="D38" t="s">
         <v>411</v>
       </c>
     </row>

</xml_diff>

<commit_message>
rerun sweet potatotes with correct yields input. tested apples country averages succesfully.
</commit_message>
<xml_diff>
--- a/data/crops/rothc_support/annual_crops_rothc_scenarios_rainfed_FAOGAEZ.xlsx
+++ b/data/crops/rothc_support/annual_crops_rothc_scenarios_rainfed_FAOGAEZ.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://worldwildlifefund-my.sharepoint.com/personal/cristobal_loyola_wwfus_org/Documents/Documents/203. Python projects/SBTN_Test/data/crops/rothc_support/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="158" documentId="8_{170725B8-9B34-4153-8604-E86F3A22CBBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{91E1FFCD-C147-47A4-AAD0-87F58580F299}"/>
+  <xr:revisionPtr revIDLastSave="163" documentId="8_{170725B8-9B34-4153-8604-E86F3A22CBBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2D470844-64B3-4BE9-BF8F-F1CC1C1366F2}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{6F94B64D-243B-49DA-AE87-045B34BFAB0F}"/>
   </bookViews>
@@ -2047,7 +2047,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2057,6 +2057,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2625,7 +2627,7 @@
         <v>344</v>
       </c>
       <c r="U2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V2" t="s">
         <v>478</v>
@@ -2691,7 +2693,7 @@
         <v>344</v>
       </c>
       <c r="U3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V3" t="s">
         <v>478</v>
@@ -2758,7 +2760,7 @@
         <v>360</v>
       </c>
       <c r="U4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V4" s="7" t="s">
         <v>478</v>
@@ -2824,7 +2826,7 @@
         <v>366</v>
       </c>
       <c r="U5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V5" s="7" t="s">
         <v>478</v>
@@ -2890,7 +2892,7 @@
         <v>369</v>
       </c>
       <c r="U6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V6" s="7" t="s">
         <v>478</v>
@@ -2956,7 +2958,7 @@
         <v>369</v>
       </c>
       <c r="U7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V7" s="7" t="s">
         <v>478</v>
@@ -3022,7 +3024,7 @@
         <v>463</v>
       </c>
       <c r="U8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V8" s="7" t="s">
         <v>478</v>
@@ -3088,7 +3090,7 @@
         <v>378</v>
       </c>
       <c r="U9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V9" s="7" t="s">
         <v>478</v>
@@ -3154,7 +3156,7 @@
         <v>378</v>
       </c>
       <c r="U10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V10" s="7" t="s">
         <v>478</v>
@@ -3220,7 +3222,7 @@
         <v>375</v>
       </c>
       <c r="U11" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V11" s="7" t="s">
         <v>478</v>
@@ -3286,7 +3288,7 @@
         <v>393</v>
       </c>
       <c r="U12" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V12" s="7" t="s">
         <v>478</v>
@@ -3352,7 +3354,7 @@
         <v>393</v>
       </c>
       <c r="U13" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V13" s="7" t="s">
         <v>478</v>
@@ -3418,7 +3420,7 @@
         <v>390</v>
       </c>
       <c r="U14" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V14" t="s">
         <v>478</v>
@@ -3484,7 +3486,7 @@
         <v>396</v>
       </c>
       <c r="U15" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V15" t="s">
         <v>478</v>
@@ -3550,7 +3552,7 @@
         <v>387</v>
       </c>
       <c r="U16" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V16" t="s">
         <v>478</v>
@@ -3603,17 +3605,17 @@
       <c r="P17">
         <v>100</v>
       </c>
-      <c r="Q17" s="6" t="s">
-        <v>451</v>
-      </c>
-      <c r="R17" s="3" t="s">
-        <v>452</v>
-      </c>
-      <c r="S17" s="3" t="s">
-        <v>450</v>
-      </c>
-      <c r="T17" s="6" t="s">
-        <v>451</v>
+      <c r="Q17" s="10" t="s">
+        <v>463</v>
+      </c>
+      <c r="R17" s="9" t="s">
+        <v>464</v>
+      </c>
+      <c r="S17" s="9" t="s">
+        <v>462</v>
+      </c>
+      <c r="T17" s="10" t="s">
+        <v>463</v>
       </c>
       <c r="U17" t="b">
         <v>1</v>
@@ -3682,7 +3684,7 @@
         <v>405</v>
       </c>
       <c r="U18" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V18" t="s">
         <v>478</v>
@@ -3748,7 +3750,7 @@
         <v>408</v>
       </c>
       <c r="U19" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V19" t="s">
         <v>478</v>
@@ -3814,7 +3816,7 @@
         <v>411</v>
       </c>
       <c r="U20" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V20" t="s">
         <v>478</v>
@@ -3880,7 +3882,7 @@
         <v>411</v>
       </c>
       <c r="U21" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V21" t="s">
         <v>478</v>

</xml_diff>

<commit_message>
failed at clipping with high percentile numbers
</commit_message>
<xml_diff>
--- a/data/crops/rothc_support/annual_crops_rothc_scenarios_rainfed_FAOGAEZ.xlsx
+++ b/data/crops/rothc_support/annual_crops_rothc_scenarios_rainfed_FAOGAEZ.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://worldwildlifefund-my.sharepoint.com/personal/cristobal_loyola_wwfus_org/Documents/Documents/203. Python projects/SBTN_Test/data/crops/rothc_support/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="165" documentId="8_{170725B8-9B34-4153-8604-E86F3A22CBBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{12A5A0C7-ED30-466F-AB4B-C74D396C96B6}"/>
+  <xr:revisionPtr revIDLastSave="166" documentId="8_{170725B8-9B34-4153-8604-E86F3A22CBBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{092985E5-D295-4F73-A8BC-C5D6038B53FE}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="100" windowWidth="19200" windowHeight="11180" xr2:uid="{6F94B64D-243B-49DA-AE87-045B34BFAB0F}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{6F94B64D-243B-49DA-AE87-045B34BFAB0F}"/>
   </bookViews>
   <sheets>
     <sheet name="scenarios" sheetId="1" r:id="rId1"/>
@@ -2689,7 +2689,7 @@
         <v>1</v>
       </c>
       <c r="AA2">
-        <v>99</v>
+        <v>99.5</v>
       </c>
     </row>
     <row r="3" spans="1:30" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
rerun first 4 crops from the annual list
</commit_message>
<xml_diff>
--- a/data/crops/rothc_support/annual_crops_rothc_scenarios_rainfed_FAOGAEZ.xlsx
+++ b/data/crops/rothc_support/annual_crops_rothc_scenarios_rainfed_FAOGAEZ.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://worldwildlifefund-my.sharepoint.com/personal/cristobal_loyola_wwfus_org/Documents/Documents/203. Python projects/SBTN_Test/data/crops/rothc_support/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="233" documentId="8_{170725B8-9B34-4153-8604-E86F3A22CBBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EDED3DCD-FA1B-4884-99A9-3C3A5A4EE171}"/>
+  <xr:revisionPtr revIDLastSave="235" documentId="8_{170725B8-9B34-4153-8604-E86F3A22CBBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FD913E1F-260C-429E-8D7F-E2BD4DCB155C}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{6F94B64D-243B-49DA-AE87-045B34BFAB0F}"/>
   </bookViews>
@@ -2021,7 +2021,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2034,9 +2034,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2121,13 +2118,13 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{55C0E0B5-21B5-4E14-A12B-9F865E445D80}" name="annual_crops_FAO_GAEZ_data_path" displayName="annual_crops_FAO_GAEZ_data_path" ref="A1:G31" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:G31" xr:uid="{55C0E0B5-21B5-4E14-A12B-9F865E445D80}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{D2CDBE54-7DFE-495A-8C47-0C4F483A9A36}" uniqueName="1" name="crop_name" queryTableFieldId="1" dataDxfId="6"/>
-    <tableColumn id="2" xr3:uid="{36A2073A-17B5-424E-891A-56660DA50771}" uniqueName="2" name="crop_type" queryTableFieldId="2" dataDxfId="5"/>
-    <tableColumn id="3" xr3:uid="{12B2EC26-9574-4C81-AE25-5FBA0E4D7A76}" uniqueName="3" name="crop_practice_string" queryTableFieldId="3" dataDxfId="4"/>
-    <tableColumn id="4" xr3:uid="{A981D2A3-6A91-43D2-B7DC-9361B9A8F20A}" uniqueName="4" name="lu_path" queryTableFieldId="4" dataDxfId="3"/>
-    <tableColumn id="5" xr3:uid="{B4B4350A-23D3-4A7F-98E1-A6388FB4A1FD}" uniqueName="5" name="pet_path" queryTableFieldId="5" dataDxfId="2"/>
-    <tableColumn id="7" xr3:uid="{EB04586B-94DF-4D65-A607-26B04ABC6F8D}" uniqueName="7" name="plantcover_path" queryTableFieldId="7" dataDxfId="0"/>
-    <tableColumn id="6" xr3:uid="{4DAE9F00-2A7F-4200-ADAF-52CB5C9B1A19}" uniqueName="6" name="irr_path" queryTableFieldId="6" dataDxfId="1"/>
+    <tableColumn id="1" xr3:uid="{D2CDBE54-7DFE-495A-8C47-0C4F483A9A36}" uniqueName="1" name="crop_name" queryTableFieldId="1" dataDxfId="10"/>
+    <tableColumn id="2" xr3:uid="{36A2073A-17B5-424E-891A-56660DA50771}" uniqueName="2" name="crop_type" queryTableFieldId="2" dataDxfId="9"/>
+    <tableColumn id="3" xr3:uid="{12B2EC26-9574-4C81-AE25-5FBA0E4D7A76}" uniqueName="3" name="crop_practice_string" queryTableFieldId="3" dataDxfId="8"/>
+    <tableColumn id="4" xr3:uid="{A981D2A3-6A91-43D2-B7DC-9361B9A8F20A}" uniqueName="4" name="lu_path" queryTableFieldId="4" dataDxfId="7"/>
+    <tableColumn id="5" xr3:uid="{B4B4350A-23D3-4A7F-98E1-A6388FB4A1FD}" uniqueName="5" name="pet_path" queryTableFieldId="5" dataDxfId="6"/>
+    <tableColumn id="7" xr3:uid="{EB04586B-94DF-4D65-A607-26B04ABC6F8D}" uniqueName="7" name="plantcover_path" queryTableFieldId="7" dataDxfId="5"/>
+    <tableColumn id="6" xr3:uid="{4DAE9F00-2A7F-4200-ADAF-52CB5C9B1A19}" uniqueName="6" name="irr_path" queryTableFieldId="6" dataDxfId="4"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2137,10 +2134,10 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{D4138EED-881E-411A-BC79-FB457DA6FC5D}" name="faogaez_yield_file_index__2" displayName="faogaez_yield_file_index__2" ref="A1:D38" tableType="queryTable" totalsRowShown="0">
   <autoFilter ref="A1:D38" xr:uid="{D4138EED-881E-411A-BC79-FB457DA6FC5D}"/>
   <tableColumns count="4">
-    <tableColumn id="5" xr3:uid="{3E605F29-4B62-42C4-B46E-4709285BBD84}" uniqueName="5" name="crop_name" queryTableFieldId="5" dataDxfId="10"/>
-    <tableColumn id="8" xr3:uid="{6E0A94BC-5E44-4F12-9A16-8BC520BDE6DA}" uniqueName="8" name="Total" queryTableFieldId="8" dataDxfId="9"/>
-    <tableColumn id="6" xr3:uid="{1F96D6F4-19CF-41F4-8F71-F7F45D3012FC}" uniqueName="6" name="Irrigated" queryTableFieldId="6" dataDxfId="8"/>
-    <tableColumn id="7" xr3:uid="{6C72B11B-83D3-4D0C-B671-13558C118237}" uniqueName="7" name="Rainfed" queryTableFieldId="7" dataDxfId="7"/>
+    <tableColumn id="5" xr3:uid="{3E605F29-4B62-42C4-B46E-4709285BBD84}" uniqueName="5" name="crop_name" queryTableFieldId="5" dataDxfId="3"/>
+    <tableColumn id="8" xr3:uid="{6E0A94BC-5E44-4F12-9A16-8BC520BDE6DA}" uniqueName="8" name="Total" queryTableFieldId="8" dataDxfId="2"/>
+    <tableColumn id="6" xr3:uid="{1F96D6F4-19CF-41F4-8F71-F7F45D3012FC}" uniqueName="6" name="Irrigated" queryTableFieldId="6" dataDxfId="1"/>
+    <tableColumn id="7" xr3:uid="{6C72B11B-83D3-4D0C-B671-13558C118237}" uniqueName="7" name="Rainfed" queryTableFieldId="7" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2592,13 +2589,13 @@
         <f t="shared" ref="G2:G21" si="0">+"RothC results for year 2030 for "&amp;A2&amp;"_"&amp;D2&amp;" in ton C/ha"</f>
         <v>RothC results for year 2030 for Barley_rf_ron in ton C/ha</v>
       </c>
-      <c r="H2" s="11" t="s">
+      <c r="H2" s="4" t="s">
         <v>335</v>
       </c>
-      <c r="I2" s="11" t="s">
+      <c r="I2" s="4" t="s">
         <v>336</v>
       </c>
-      <c r="J2" s="11" t="s">
+      <c r="J2" s="4" t="s">
         <v>337</v>
       </c>
       <c r="N2" t="b">
@@ -2670,13 +2667,13 @@
         <f t="shared" si="0"/>
         <v>RothC results for year 2030 for Barley_rf_roff in ton C/ha</v>
       </c>
-      <c r="H3" s="11" t="s">
+      <c r="H3" s="4" t="s">
         <v>335</v>
       </c>
-      <c r="I3" s="11" t="s">
+      <c r="I3" s="4" t="s">
         <v>336</v>
       </c>
-      <c r="J3" s="11" t="s">
+      <c r="J3" s="4" t="s">
         <v>337</v>
       </c>
       <c r="N3" t="b">
@@ -2748,13 +2745,13 @@
         <f t="shared" si="0"/>
         <v>RothC results for year 2030 for Cotton_rf in ton C/ha</v>
       </c>
-      <c r="H4" s="12" t="s">
+      <c r="H4" s="3" t="s">
         <v>478</v>
       </c>
-      <c r="I4" s="12" t="s">
+      <c r="I4" s="3" t="s">
         <v>479</v>
       </c>
-      <c r="J4" s="12" t="s">
+      <c r="J4" s="3" t="s">
         <v>480</v>
       </c>
       <c r="K4" s="6"/>
@@ -2827,13 +2824,13 @@
         <f t="shared" si="0"/>
         <v>RothC results for year 2030 for Groundnut_rf in ton C/ha</v>
       </c>
-      <c r="H5" s="12" t="s">
+      <c r="H5" s="3" t="s">
         <v>481</v>
       </c>
-      <c r="I5" s="12" t="s">
+      <c r="I5" s="3" t="s">
         <v>482</v>
       </c>
-      <c r="J5" s="12" t="s">
+      <c r="J5" s="3" t="s">
         <v>483</v>
       </c>
       <c r="K5" s="6"/>
@@ -2906,13 +2903,13 @@
         <f t="shared" si="0"/>
         <v>RothC results for year 2030 for Maize_rf_ron in ton C/ha</v>
       </c>
-      <c r="H6" s="11" t="s">
+      <c r="H6" s="4" t="s">
         <v>484</v>
       </c>
-      <c r="I6" s="11" t="s">
+      <c r="I6" s="4" t="s">
         <v>485</v>
       </c>
-      <c r="J6" s="11" t="s">
+      <c r="J6" s="4" t="s">
         <v>486</v>
       </c>
       <c r="N6" t="b">
@@ -2937,7 +2934,7 @@
         <v>368</v>
       </c>
       <c r="U6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V6" s="7" t="s">
         <v>477</v>
@@ -2984,13 +2981,13 @@
         <f t="shared" si="0"/>
         <v>RothC results for year 2030 for Maize_rf_roff in ton C/ha</v>
       </c>
-      <c r="H7" s="11" t="s">
+      <c r="H7" s="4" t="s">
         <v>484</v>
       </c>
-      <c r="I7" s="11" t="s">
+      <c r="I7" s="4" t="s">
         <v>485</v>
       </c>
-      <c r="J7" s="11" t="s">
+      <c r="J7" s="4" t="s">
         <v>486</v>
       </c>
       <c r="N7" t="b">
@@ -3015,7 +3012,7 @@
         <v>368</v>
       </c>
       <c r="U7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V7" s="7" t="s">
         <v>477</v>
@@ -3062,13 +3059,13 @@
         <f t="shared" si="0"/>
         <v>RothC results for year 2030 for Potato_rf in ton C/ha</v>
       </c>
-      <c r="H8" s="12" t="s">
+      <c r="H8" s="3" t="s">
         <v>487</v>
       </c>
-      <c r="I8" s="12" t="s">
+      <c r="I8" s="3" t="s">
         <v>488</v>
       </c>
-      <c r="J8" s="12" t="s">
+      <c r="J8" s="3" t="s">
         <v>489</v>
       </c>
       <c r="N8" t="b">
@@ -3093,7 +3090,7 @@
         <v>462</v>
       </c>
       <c r="U8" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V8" s="7" t="s">
         <v>477</v>
@@ -3140,13 +3137,13 @@
         <f t="shared" si="0"/>
         <v>RothC results for year 2030 for Rapeseed_rf_ron in ton C/ha</v>
       </c>
-      <c r="H9" s="11" t="s">
+      <c r="H9" s="4" t="s">
         <v>490</v>
       </c>
-      <c r="I9" s="11" t="s">
+      <c r="I9" s="4" t="s">
         <v>491</v>
       </c>
-      <c r="J9" s="11" t="s">
+      <c r="J9" s="4" t="s">
         <v>492</v>
       </c>
       <c r="N9" t="b">
@@ -3171,7 +3168,7 @@
         <v>377</v>
       </c>
       <c r="U9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V9" s="7" t="s">
         <v>477</v>
@@ -3218,13 +3215,13 @@
         <f t="shared" si="0"/>
         <v>RothC results for year 2030 for Rapeseed_rf_roff in ton C/ha</v>
       </c>
-      <c r="H10" s="11" t="s">
+      <c r="H10" s="4" t="s">
         <v>490</v>
       </c>
-      <c r="I10" s="11" t="s">
+      <c r="I10" s="4" t="s">
         <v>491</v>
       </c>
-      <c r="J10" s="11" t="s">
+      <c r="J10" s="4" t="s">
         <v>492</v>
       </c>
       <c r="N10" t="b">
@@ -3249,7 +3246,7 @@
         <v>377</v>
       </c>
       <c r="U10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V10" s="7" t="s">
         <v>477</v>
@@ -3327,7 +3324,7 @@
         <v>374</v>
       </c>
       <c r="U11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V11" s="7" t="s">
         <v>477</v>
@@ -3374,13 +3371,13 @@
         <f t="shared" si="0"/>
         <v>RothC results for year 2030 for Sorghum_rf_ron in ton C/ha</v>
       </c>
-      <c r="H12" s="11" t="s">
+      <c r="H12" s="4" t="s">
         <v>599</v>
       </c>
-      <c r="I12" s="11" t="s">
+      <c r="I12" s="4" t="s">
         <v>600</v>
       </c>
-      <c r="J12" s="11" t="s">
+      <c r="J12" s="4" t="s">
         <v>601</v>
       </c>
       <c r="N12" t="b">
@@ -3405,7 +3402,7 @@
         <v>392</v>
       </c>
       <c r="U12" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V12" s="7" t="s">
         <v>477</v>
@@ -3452,13 +3449,13 @@
         <f t="shared" si="0"/>
         <v>RothC results for year 2030 for Sorghum_rf_roff in ton C/ha</v>
       </c>
-      <c r="H13" s="11" t="s">
+      <c r="H13" s="4" t="s">
         <v>599</v>
       </c>
-      <c r="I13" s="11" t="s">
+      <c r="I13" s="4" t="s">
         <v>600</v>
       </c>
-      <c r="J13" s="11" t="s">
+      <c r="J13" s="4" t="s">
         <v>601</v>
       </c>
       <c r="N13" t="b">
@@ -3483,7 +3480,7 @@
         <v>392</v>
       </c>
       <c r="U13" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V13" s="7" t="s">
         <v>477</v>
@@ -3530,13 +3527,13 @@
         <f t="shared" si="0"/>
         <v>RothC results for year 2030 for Soybean_rf in ton C/ha</v>
       </c>
-      <c r="H14" s="12" t="s">
+      <c r="H14" s="3" t="s">
         <v>493</v>
       </c>
-      <c r="I14" s="12" t="s">
+      <c r="I14" s="3" t="s">
         <v>494</v>
       </c>
-      <c r="J14" s="12" t="s">
+      <c r="J14" s="3" t="s">
         <v>495</v>
       </c>
       <c r="N14" t="b">
@@ -3561,7 +3558,7 @@
         <v>389</v>
       </c>
       <c r="U14" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V14" t="s">
         <v>477</v>
@@ -3639,7 +3636,7 @@
         <v>395</v>
       </c>
       <c r="U15" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V15" t="s">
         <v>477</v>
@@ -3686,13 +3683,13 @@
         <f t="shared" si="0"/>
         <v>RothC results for year 2030 for Sunflower_rf in ton C/ha</v>
       </c>
-      <c r="H16" s="11" t="s">
+      <c r="H16" s="4" t="s">
         <v>567</v>
       </c>
-      <c r="I16" s="11" t="s">
+      <c r="I16" s="4" t="s">
         <v>568</v>
       </c>
-      <c r="J16" s="11" t="s">
+      <c r="J16" s="4" t="s">
         <v>569</v>
       </c>
       <c r="N16" t="b">
@@ -3717,7 +3714,7 @@
         <v>386</v>
       </c>
       <c r="U16" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V16" t="s">
         <v>477</v>
@@ -3764,13 +3761,13 @@
         <f t="shared" si="0"/>
         <v>RothC results for year 2030 for Sweet potato_rf in ton C/ha</v>
       </c>
-      <c r="H17" s="12" t="s">
+      <c r="H17" s="3" t="s">
         <v>570</v>
       </c>
-      <c r="I17" s="12" t="s">
+      <c r="I17" s="3" t="s">
         <v>571</v>
       </c>
-      <c r="J17" s="12" t="s">
+      <c r="J17" s="3" t="s">
         <v>572</v>
       </c>
       <c r="N17" t="b">
@@ -3795,7 +3792,7 @@
         <v>462</v>
       </c>
       <c r="U17" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V17" t="s">
         <v>477</v>
@@ -3842,13 +3839,13 @@
         <f t="shared" si="0"/>
         <v>RothC results for year 2030 for Tobacco_rf in ton C/ha</v>
       </c>
-      <c r="H18" s="11" t="s">
+      <c r="H18" s="4" t="s">
         <v>573</v>
       </c>
-      <c r="I18" s="11" t="s">
+      <c r="I18" s="4" t="s">
         <v>574</v>
       </c>
-      <c r="J18" s="11" t="s">
+      <c r="J18" s="4" t="s">
         <v>575</v>
       </c>
       <c r="N18" t="b">
@@ -3873,7 +3870,7 @@
         <v>404</v>
       </c>
       <c r="U18" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V18" t="s">
         <v>477</v>
@@ -3920,13 +3917,13 @@
         <f t="shared" si="0"/>
         <v>RothC results for year 2030 for Tomato_rf in ton C/ha</v>
       </c>
-      <c r="H19" s="12" t="s">
+      <c r="H19" s="3" t="s">
         <v>576</v>
       </c>
-      <c r="I19" s="12" t="s">
+      <c r="I19" s="3" t="s">
         <v>577</v>
       </c>
-      <c r="J19" s="12" t="s">
+      <c r="J19" s="3" t="s">
         <v>578</v>
       </c>
       <c r="N19" t="b">
@@ -3951,7 +3948,7 @@
         <v>407</v>
       </c>
       <c r="U19" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V19" t="s">
         <v>477</v>
@@ -3998,13 +3995,13 @@
         <f t="shared" si="0"/>
         <v>RothC results for year 2030 for Wheat_rf_ron in ton C/ha</v>
       </c>
-      <c r="H20" s="11" t="s">
+      <c r="H20" s="4" t="s">
         <v>579</v>
       </c>
-      <c r="I20" s="11" t="s">
+      <c r="I20" s="4" t="s">
         <v>580</v>
       </c>
-      <c r="J20" s="11" t="s">
+      <c r="J20" s="4" t="s">
         <v>581</v>
       </c>
       <c r="N20" t="b">
@@ -4029,7 +4026,7 @@
         <v>410</v>
       </c>
       <c r="U20" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V20" t="s">
         <v>477</v>
@@ -4076,13 +4073,13 @@
         <f t="shared" si="0"/>
         <v>RothC results for year 2030 for Wheat_rf_roff in ton C/ha</v>
       </c>
-      <c r="H21" s="11" t="s">
+      <c r="H21" s="4" t="s">
         <v>579</v>
       </c>
-      <c r="I21" s="11" t="s">
+      <c r="I21" s="4" t="s">
         <v>580</v>
       </c>
-      <c r="J21" s="11" t="s">
+      <c r="J21" s="4" t="s">
         <v>581</v>
       </c>
       <c r="N21" t="b">
@@ -4107,7 +4104,7 @@
         <v>410</v>
       </c>
       <c r="U21" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V21" t="s">
         <v>477</v>
@@ -4176,692 +4173,692 @@
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A2" s="10" t="s">
+      <c r="A2" t="s">
         <v>15</v>
       </c>
-      <c r="B2" s="10" t="s">
+      <c r="B2" t="s">
         <v>502</v>
       </c>
-      <c r="C2" s="10" t="s">
+      <c r="C2" t="s">
         <v>503</v>
       </c>
-      <c r="D2" s="10" t="s">
+      <c r="D2" t="s">
         <v>334</v>
       </c>
-      <c r="E2" s="10" t="s">
+      <c r="E2" t="s">
         <v>504</v>
       </c>
-      <c r="F2" s="10" t="s">
+      <c r="F2" t="s">
         <v>506</v>
       </c>
-      <c r="G2" s="10" t="s">
+      <c r="G2" t="s">
         <v>505</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A3" s="10" t="s">
+      <c r="A3" t="s">
         <v>16</v>
       </c>
-      <c r="B3" s="10" t="s">
+      <c r="B3" t="s">
         <v>502</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="C3" t="s">
         <v>507</v>
       </c>
-      <c r="D3" s="10" t="s">
+      <c r="D3" t="s">
         <v>508</v>
       </c>
-      <c r="E3" s="10" t="s">
+      <c r="E3" t="s">
         <v>509</v>
       </c>
-      <c r="F3" s="10" t="s">
+      <c r="F3" t="s">
         <v>511</v>
       </c>
-      <c r="G3" s="10" t="s">
+      <c r="G3" t="s">
         <v>510</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A4" s="10" t="s">
+      <c r="A4" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="10" t="s">
+      <c r="B4" t="s">
         <v>502</v>
       </c>
-      <c r="C4" s="10" t="s">
+      <c r="C4" t="s">
         <v>507</v>
       </c>
-      <c r="D4" s="10" t="s">
+      <c r="D4" t="s">
         <v>512</v>
       </c>
-      <c r="E4" s="10" t="s">
+      <c r="E4" t="s">
         <v>513</v>
       </c>
-      <c r="F4" s="10" t="s">
+      <c r="F4" t="s">
         <v>515</v>
       </c>
-      <c r="G4" s="10" t="s">
+      <c r="G4" t="s">
         <v>514</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A5" s="10" t="s">
+      <c r="A5" t="s">
         <v>18</v>
       </c>
-      <c r="B5" s="10" t="s">
+      <c r="B5" t="s">
         <v>502</v>
       </c>
-      <c r="C5" s="10" t="s">
+      <c r="C5" t="s">
         <v>507</v>
       </c>
-      <c r="D5" s="10" t="s">
+      <c r="D5" t="s">
         <v>516</v>
       </c>
-      <c r="E5" s="10" t="s">
+      <c r="E5" t="s">
         <v>517</v>
       </c>
-      <c r="F5" s="10" t="s">
+      <c r="F5" t="s">
         <v>519</v>
       </c>
-      <c r="G5" s="10" t="s">
+      <c r="G5" t="s">
         <v>518</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A6" s="10" t="s">
+      <c r="A6" t="s">
         <v>20</v>
       </c>
-      <c r="B6" s="10" t="s">
+      <c r="B6" t="s">
         <v>502</v>
       </c>
-      <c r="C6" s="10" t="s">
+      <c r="C6" t="s">
         <v>503</v>
       </c>
-      <c r="D6" s="10" t="s">
+      <c r="D6" t="s">
         <v>520</v>
       </c>
-      <c r="E6" s="10" t="s">
+      <c r="E6" t="s">
         <v>521</v>
       </c>
-      <c r="F6" s="10" t="s">
+      <c r="F6" t="s">
         <v>523</v>
       </c>
-      <c r="G6" s="10" t="s">
+      <c r="G6" t="s">
         <v>522</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A7" s="10" t="s">
+      <c r="A7" t="s">
         <v>21</v>
       </c>
-      <c r="B7" s="10" t="s">
+      <c r="B7" t="s">
         <v>502</v>
       </c>
-      <c r="C7" s="10" t="s">
+      <c r="C7" t="s">
         <v>507</v>
       </c>
-      <c r="D7" s="10" t="s">
+      <c r="D7" t="s">
         <v>524</v>
       </c>
-      <c r="E7" s="10" t="s">
+      <c r="E7" t="s">
         <v>525</v>
       </c>
-      <c r="F7" s="10" t="s">
+      <c r="F7" t="s">
         <v>527</v>
       </c>
-      <c r="G7" s="10" t="s">
+      <c r="G7" t="s">
         <v>526</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A8" s="10" t="s">
+      <c r="A8" t="s">
         <v>22</v>
       </c>
-      <c r="B8" s="10" t="s">
+      <c r="B8" t="s">
         <v>502</v>
       </c>
-      <c r="C8" s="10" t="s">
+      <c r="C8" t="s">
         <v>507</v>
       </c>
-      <c r="D8" s="10" t="s">
+      <c r="D8" t="s">
         <v>528</v>
       </c>
-      <c r="E8" s="10" t="s">
+      <c r="E8" t="s">
         <v>529</v>
       </c>
-      <c r="F8" s="10" t="s">
+      <c r="F8" t="s">
         <v>531</v>
       </c>
-      <c r="G8" s="10" t="s">
+      <c r="G8" t="s">
         <v>530</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A9" s="10" t="s">
+      <c r="A9" t="s">
         <v>23</v>
       </c>
-      <c r="B9" s="10" t="s">
+      <c r="B9" t="s">
         <v>502</v>
       </c>
-      <c r="C9" s="10" t="s">
+      <c r="C9" t="s">
         <v>503</v>
       </c>
-      <c r="D9" s="10" t="s">
+      <c r="D9" t="s">
         <v>532</v>
       </c>
-      <c r="E9" s="10" t="s">
+      <c r="E9" t="s">
         <v>533</v>
       </c>
-      <c r="F9" s="10" t="s">
+      <c r="F9" t="s">
         <v>535</v>
       </c>
-      <c r="G9" s="10" t="s">
+      <c r="G9" t="s">
         <v>534</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A10" s="10" t="s">
+      <c r="A10" t="s">
         <v>25</v>
       </c>
-      <c r="B10" s="10" t="s">
+      <c r="B10" t="s">
         <v>502</v>
       </c>
-      <c r="C10" s="10" t="s">
+      <c r="C10" t="s">
         <v>503</v>
       </c>
-      <c r="D10" s="10" t="s">
+      <c r="D10" t="s">
         <v>536</v>
       </c>
-      <c r="E10" s="10" t="s">
+      <c r="E10" t="s">
         <v>537</v>
       </c>
-      <c r="F10" s="10" t="s">
+      <c r="F10" t="s">
         <v>539</v>
       </c>
-      <c r="G10" s="10" t="s">
+      <c r="G10" t="s">
         <v>538</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A11" s="10" t="s">
+      <c r="A11" t="s">
         <v>26</v>
       </c>
-      <c r="B11" s="10" t="s">
+      <c r="B11" t="s">
         <v>502</v>
       </c>
-      <c r="C11" s="10" t="s">
+      <c r="C11" t="s">
         <v>507</v>
       </c>
-      <c r="D11" s="10" t="s">
+      <c r="D11" t="s">
         <v>540</v>
       </c>
-      <c r="E11" s="10" t="s">
+      <c r="E11" t="s">
         <v>541</v>
       </c>
-      <c r="F11" s="10" t="s">
+      <c r="F11" t="s">
         <v>543</v>
       </c>
-      <c r="G11" s="10" t="s">
+      <c r="G11" t="s">
         <v>542</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A12" s="10" t="s">
+      <c r="A12" t="s">
         <v>27</v>
       </c>
-      <c r="B12" s="10" t="s">
+      <c r="B12" t="s">
         <v>502</v>
       </c>
-      <c r="C12" s="10" t="s">
+      <c r="C12" t="s">
         <v>507</v>
       </c>
-      <c r="D12" s="10" t="s">
+      <c r="D12" t="s">
         <v>544</v>
       </c>
-      <c r="E12" s="10" t="s">
+      <c r="E12" t="s">
         <v>545</v>
       </c>
-      <c r="F12" s="10" t="s">
+      <c r="F12" t="s">
         <v>547</v>
       </c>
-      <c r="G12" s="10" t="s">
+      <c r="G12" t="s">
         <v>546</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A13" s="10" t="s">
+      <c r="A13" t="s">
         <v>29</v>
       </c>
-      <c r="B13" s="10" t="s">
+      <c r="B13" t="s">
         <v>502</v>
       </c>
-      <c r="C13" s="10" t="s">
+      <c r="C13" t="s">
         <v>507</v>
       </c>
-      <c r="D13" s="10" t="s">
+      <c r="D13" t="s">
         <v>548</v>
       </c>
-      <c r="E13" s="10" t="s">
+      <c r="E13" t="s">
         <v>549</v>
       </c>
-      <c r="F13" s="10" t="s">
+      <c r="F13" t="s">
         <v>551</v>
       </c>
-      <c r="G13" s="10" t="s">
+      <c r="G13" t="s">
         <v>550</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A14" s="10" t="s">
+      <c r="A14" t="s">
         <v>30</v>
       </c>
-      <c r="B14" s="10" t="s">
+      <c r="B14" t="s">
         <v>502</v>
       </c>
-      <c r="C14" s="10" t="s">
+      <c r="C14" t="s">
         <v>507</v>
       </c>
-      <c r="D14" s="10" t="s">
+      <c r="D14" t="s">
         <v>552</v>
       </c>
-      <c r="E14" s="10" t="s">
+      <c r="E14" t="s">
         <v>553</v>
       </c>
-      <c r="F14" s="10" t="s">
+      <c r="F14" t="s">
         <v>555</v>
       </c>
-      <c r="G14" s="10" t="s">
+      <c r="G14" t="s">
         <v>554</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A15" s="10" t="s">
+      <c r="A15" t="s">
         <v>31</v>
       </c>
-      <c r="B15" s="10" t="s">
+      <c r="B15" t="s">
         <v>502</v>
       </c>
-      <c r="C15" s="10" t="s">
+      <c r="C15" t="s">
         <v>507</v>
       </c>
-      <c r="D15" s="10" t="s">
+      <c r="D15" t="s">
         <v>556</v>
       </c>
-      <c r="E15" s="10" t="s">
+      <c r="E15" t="s">
         <v>557</v>
       </c>
-      <c r="F15" s="10" t="s">
+      <c r="F15" t="s">
         <v>559</v>
       </c>
-      <c r="G15" s="10" t="s">
+      <c r="G15" t="s">
         <v>558</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A16" s="10" t="s">
+      <c r="A16" t="s">
         <v>32</v>
       </c>
-      <c r="B16" s="10" t="s">
+      <c r="B16" t="s">
         <v>502</v>
       </c>
-      <c r="C16" s="10" t="s">
+      <c r="C16" t="s">
         <v>507</v>
       </c>
-      <c r="D16" s="10" t="s">
+      <c r="D16" t="s">
         <v>560</v>
       </c>
-      <c r="E16" s="10" t="s">
+      <c r="E16" t="s">
         <v>561</v>
       </c>
-      <c r="F16" s="10" t="s">
+      <c r="F16" t="s">
         <v>563</v>
       </c>
-      <c r="G16" s="10" t="s">
+      <c r="G16" t="s">
         <v>562</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A17" s="10" t="s">
+      <c r="A17" t="s">
         <v>33</v>
       </c>
-      <c r="B17" s="10" t="s">
+      <c r="B17" t="s">
         <v>502</v>
       </c>
-      <c r="C17" s="10" t="s">
+      <c r="C17" t="s">
         <v>503</v>
       </c>
-      <c r="D17" s="10" t="s">
+      <c r="D17" t="s">
         <v>586</v>
       </c>
-      <c r="E17" s="10" t="s">
+      <c r="E17" t="s">
         <v>564</v>
       </c>
-      <c r="F17" s="10" t="s">
+      <c r="F17" t="s">
         <v>566</v>
       </c>
-      <c r="G17" s="10" t="s">
+      <c r="G17" t="s">
         <v>565</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A18" s="10" t="s">
+      <c r="A18" t="s">
         <v>15</v>
       </c>
-      <c r="B18" s="10" t="s">
+      <c r="B18" t="s">
         <v>502</v>
       </c>
-      <c r="C18" s="10" t="s">
+      <c r="C18" t="s">
         <v>35</v>
       </c>
-      <c r="D18" s="10" t="s">
+      <c r="D18" t="s">
         <v>335</v>
       </c>
-      <c r="E18" s="10" t="s">
+      <c r="E18" t="s">
         <v>336</v>
       </c>
-      <c r="F18" s="10" t="s">
+      <c r="F18" t="s">
         <v>337</v>
       </c>
-      <c r="G18" s="10" t="s">
+      <c r="G18" t="s">
         <v>345</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A19" s="10" t="s">
+      <c r="A19" t="s">
         <v>18</v>
       </c>
-      <c r="B19" s="10" t="s">
+      <c r="B19" t="s">
         <v>502</v>
       </c>
-      <c r="C19" s="10" t="s">
+      <c r="C19" t="s">
         <v>37</v>
       </c>
-      <c r="D19" s="10" t="s">
+      <c r="D19" t="s">
         <v>478</v>
       </c>
-      <c r="E19" s="10" t="s">
+      <c r="E19" t="s">
         <v>479</v>
       </c>
-      <c r="F19" s="10" t="s">
+      <c r="F19" t="s">
         <v>480</v>
       </c>
-      <c r="G19" s="10" t="s">
+      <c r="G19" t="s">
         <v>345</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A20" s="10" t="s">
+      <c r="A20" t="s">
         <v>20</v>
       </c>
-      <c r="B20" s="10" t="s">
+      <c r="B20" t="s">
         <v>502</v>
       </c>
-      <c r="C20" s="10" t="s">
+      <c r="C20" t="s">
         <v>35</v>
       </c>
-      <c r="D20" s="10" t="s">
+      <c r="D20" t="s">
         <v>484</v>
       </c>
-      <c r="E20" s="10" t="s">
+      <c r="E20" t="s">
         <v>485</v>
       </c>
-      <c r="F20" s="10" t="s">
+      <c r="F20" t="s">
         <v>486</v>
       </c>
-      <c r="G20" s="10" t="s">
+      <c r="G20" t="s">
         <v>345</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A21" s="10" t="s">
+      <c r="A21" t="s">
         <v>22</v>
       </c>
-      <c r="B21" s="10" t="s">
+      <c r="B21" t="s">
         <v>502</v>
       </c>
-      <c r="C21" s="10" t="s">
+      <c r="C21" t="s">
         <v>37</v>
       </c>
-      <c r="D21" s="10" t="s">
+      <c r="D21" t="s">
         <v>487</v>
       </c>
-      <c r="E21" s="10" t="s">
+      <c r="E21" t="s">
         <v>488</v>
       </c>
-      <c r="F21" s="10" t="s">
+      <c r="F21" t="s">
         <v>489</v>
       </c>
-      <c r="G21" s="10" t="s">
+      <c r="G21" t="s">
         <v>345</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A22" s="10" t="s">
+      <c r="A22" t="s">
         <v>23</v>
       </c>
-      <c r="B22" s="10" t="s">
+      <c r="B22" t="s">
         <v>502</v>
       </c>
-      <c r="C22" s="10" t="s">
+      <c r="C22" t="s">
         <v>35</v>
       </c>
-      <c r="D22" s="10" t="s">
+      <c r="D22" t="s">
         <v>490</v>
       </c>
-      <c r="E22" s="10" t="s">
+      <c r="E22" t="s">
         <v>491</v>
       </c>
-      <c r="F22" s="10" t="s">
+      <c r="F22" t="s">
         <v>492</v>
       </c>
-      <c r="G22" s="10" t="s">
+      <c r="G22" t="s">
         <v>345</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A23" s="10" t="s">
+      <c r="A23" t="s">
         <v>26</v>
       </c>
-      <c r="B23" s="10" t="s">
+      <c r="B23" t="s">
         <v>502</v>
       </c>
-      <c r="C23" s="10" t="s">
+      <c r="C23" t="s">
         <v>37</v>
       </c>
-      <c r="D23" s="10" t="s">
+      <c r="D23" t="s">
         <v>493</v>
       </c>
-      <c r="E23" s="10" t="s">
+      <c r="E23" t="s">
         <v>494</v>
       </c>
-      <c r="F23" s="10" t="s">
+      <c r="F23" t="s">
         <v>495</v>
       </c>
-      <c r="G23" s="10" t="s">
+      <c r="G23" t="s">
         <v>345</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A24" s="10" t="s">
+      <c r="A24" t="s">
         <v>29</v>
       </c>
-      <c r="B24" s="10" t="s">
+      <c r="B24" t="s">
         <v>502</v>
       </c>
-      <c r="C24" s="10" t="s">
+      <c r="C24" t="s">
         <v>37</v>
       </c>
-      <c r="D24" s="10" t="s">
+      <c r="D24" t="s">
         <v>567</v>
       </c>
-      <c r="E24" s="10" t="s">
+      <c r="E24" t="s">
         <v>568</v>
       </c>
-      <c r="F24" s="10" t="s">
+      <c r="F24" t="s">
         <v>569</v>
       </c>
-      <c r="G24" s="10" t="s">
+      <c r="G24" t="s">
         <v>345</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A25" s="10" t="s">
+      <c r="A25" t="s">
         <v>30</v>
       </c>
-      <c r="B25" s="10" t="s">
+      <c r="B25" t="s">
         <v>502</v>
       </c>
-      <c r="C25" s="10" t="s">
+      <c r="C25" t="s">
         <v>37</v>
       </c>
-      <c r="D25" s="10" t="s">
+      <c r="D25" t="s">
         <v>570</v>
       </c>
-      <c r="E25" s="10" t="s">
+      <c r="E25" t="s">
         <v>571</v>
       </c>
-      <c r="F25" s="10" t="s">
+      <c r="F25" t="s">
         <v>572</v>
       </c>
-      <c r="G25" s="10" t="s">
+      <c r="G25" t="s">
         <v>345</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A26" s="10" t="s">
+      <c r="A26" t="s">
         <v>31</v>
       </c>
-      <c r="B26" s="10" t="s">
+      <c r="B26" t="s">
         <v>502</v>
       </c>
-      <c r="C26" s="10" t="s">
+      <c r="C26" t="s">
         <v>37</v>
       </c>
-      <c r="D26" s="10" t="s">
+      <c r="D26" t="s">
         <v>573</v>
       </c>
-      <c r="E26" s="10" t="s">
+      <c r="E26" t="s">
         <v>574</v>
       </c>
-      <c r="F26" s="10" t="s">
+      <c r="F26" t="s">
         <v>575</v>
       </c>
-      <c r="G26" s="10" t="s">
+      <c r="G26" t="s">
         <v>345</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A27" s="10" t="s">
+      <c r="A27" t="s">
         <v>32</v>
       </c>
-      <c r="B27" s="10" t="s">
+      <c r="B27" t="s">
         <v>502</v>
       </c>
-      <c r="C27" s="10" t="s">
+      <c r="C27" t="s">
         <v>37</v>
       </c>
-      <c r="D27" s="10" t="s">
+      <c r="D27" t="s">
         <v>576</v>
       </c>
-      <c r="E27" s="10" t="s">
+      <c r="E27" t="s">
         <v>577</v>
       </c>
-      <c r="F27" s="10" t="s">
+      <c r="F27" t="s">
         <v>578</v>
       </c>
-      <c r="G27" s="10" t="s">
+      <c r="G27" t="s">
         <v>345</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A28" s="10" t="s">
+      <c r="A28" t="s">
         <v>33</v>
       </c>
-      <c r="B28" s="10" t="s">
+      <c r="B28" t="s">
         <v>502</v>
       </c>
-      <c r="C28" s="10" t="s">
+      <c r="C28" t="s">
         <v>35</v>
       </c>
-      <c r="D28" s="10" t="s">
+      <c r="D28" t="s">
         <v>579</v>
       </c>
-      <c r="E28" s="10" t="s">
+      <c r="E28" t="s">
         <v>580</v>
       </c>
-      <c r="F28" s="10" t="s">
+      <c r="F28" t="s">
         <v>581</v>
       </c>
-      <c r="G28" s="10" t="s">
+      <c r="G28" t="s">
         <v>345</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A29" s="10" t="s">
+      <c r="A29" t="s">
         <v>19</v>
       </c>
-      <c r="B29" s="10" t="s">
+      <c r="B29" t="s">
         <v>502</v>
       </c>
-      <c r="C29" s="10" t="s">
+      <c r="C29" t="s">
         <v>507</v>
       </c>
-      <c r="D29" s="10" t="s">
+      <c r="D29" t="s">
         <v>582</v>
       </c>
-      <c r="E29" s="10" t="s">
+      <c r="E29" t="s">
         <v>583</v>
       </c>
-      <c r="F29" s="10" t="s">
+      <c r="F29" t="s">
         <v>585</v>
       </c>
-      <c r="G29" s="10" t="s">
+      <c r="G29" t="s">
         <v>584</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A30" s="10" t="s">
+      <c r="A30" t="s">
         <v>19</v>
       </c>
-      <c r="B30" s="10" t="s">
+      <c r="B30" t="s">
         <v>502</v>
       </c>
-      <c r="C30" s="10" t="s">
+      <c r="C30" t="s">
         <v>37</v>
       </c>
-      <c r="D30" s="10" t="s">
+      <c r="D30" t="s">
         <v>481</v>
       </c>
-      <c r="E30" s="10" t="s">
+      <c r="E30" t="s">
         <v>482</v>
       </c>
-      <c r="F30" s="10" t="s">
+      <c r="F30" t="s">
         <v>483</v>
       </c>
-      <c r="G30" s="10" t="s">
+      <c r="G30" t="s">
         <v>345</v>
       </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A31" s="10" t="s">
+      <c r="A31" t="s">
         <v>25</v>
       </c>
-      <c r="B31" s="10" t="s">
+      <c r="B31" t="s">
         <v>502</v>
       </c>
-      <c r="C31" s="10" t="s">
+      <c r="C31" t="s">
         <v>35</v>
       </c>
-      <c r="D31" s="10" t="s">
+      <c r="D31" t="s">
         <v>599</v>
       </c>
-      <c r="E31" s="10" t="s">
+      <c r="E31" t="s">
         <v>600</v>
       </c>
-      <c r="F31" s="10" t="s">
+      <c r="F31" t="s">
         <v>601</v>
       </c>
-      <c r="G31" s="10" t="s">
+      <c r="G31" t="s">
         <v>345</v>
       </c>
     </row>

</xml_diff>